<commit_message>
fixing and testing the economic cost objective
</commit_message>
<xml_diff>
--- a/tests/optim_results_stillbirths.xlsx
+++ b/tests/optim_results_stillbirths.xlsx
@@ -202,6 +202,9 @@
     <t>Total (discounted)</t>
   </si>
   <si>
+    <t>Total economic cost (discounted)</t>
+  </si>
+  <si>
     <t>Economic cost of child deaths (discounted)</t>
   </si>
   <si>
@@ -224,9 +227,6 @@
   </si>
   <si>
     <t>Economic cost of maternal anemia (discounted)</t>
-  </si>
-  <si>
-    <t>Total economic cost (discounted)</t>
   </si>
 </sst>
 </file>
@@ -6974,46 +6974,46 @@
         <v>0</v>
       </c>
       <c r="E2" s="3">
-        <v>22757201772.49164</v>
+        <v>85541470193.56918</v>
       </c>
       <c r="F2" s="3">
-        <v>23044218247.92232</v>
+        <v>86187427554.35443</v>
       </c>
       <c r="G2" s="3">
-        <v>23403635503.35503</v>
+        <v>86922452051.73706</v>
       </c>
       <c r="H2" s="3">
-        <v>23792304871.19622</v>
+        <v>87761170616.90669</v>
       </c>
       <c r="I2" s="3">
-        <v>24255816995.93973</v>
+        <v>88849114804.09862</v>
       </c>
       <c r="J2" s="3">
-        <v>24751863662.06786</v>
+        <v>90148703432.2594</v>
       </c>
       <c r="K2" s="3">
-        <v>25208854936.40596</v>
+        <v>91569937596.81255</v>
       </c>
       <c r="L2" s="3">
-        <v>25784538829.65731</v>
+        <v>93269797963.53577</v>
       </c>
       <c r="M2" s="3">
-        <v>26331534604.66109</v>
+        <v>95042342452.73726</v>
       </c>
       <c r="N2" s="3">
-        <v>26886612327.6869</v>
+        <v>96928156285.89066</v>
       </c>
       <c r="O2" s="3">
-        <v>27440386767.30297</v>
+        <v>98893365824.02509</v>
       </c>
       <c r="P2" s="3">
-        <v>28059933837.37794</v>
+        <v>100989432623.0793</v>
       </c>
       <c r="Q2" s="3">
-        <v>28637527708.94907</v>
+        <v>103082693291.142</v>
       </c>
       <c r="R2" s="3">
-        <v>330354430065.014</v>
+        <v>1205186064690.148</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -7030,46 +7030,46 @@
         <v>0</v>
       </c>
       <c r="E3" s="3">
-        <v>2824673820.668513</v>
+        <v>22757201772.49164</v>
       </c>
       <c r="F3" s="3">
-        <v>2892132503.559748</v>
+        <v>23044218247.92232</v>
       </c>
       <c r="G3" s="3">
-        <v>2945073514.468478</v>
+        <v>23403635503.35503</v>
       </c>
       <c r="H3" s="3">
-        <v>2997153077.667239</v>
+        <v>23792304871.19622</v>
       </c>
       <c r="I3" s="3">
-        <v>3062818764.410106</v>
+        <v>24255816995.93973</v>
       </c>
       <c r="J3" s="3">
-        <v>3128885547.708316</v>
+        <v>24751863662.06786</v>
       </c>
       <c r="K3" s="3">
-        <v>3181383526.957898</v>
+        <v>25208854936.40596</v>
       </c>
       <c r="L3" s="3">
-        <v>3259792881.108632</v>
+        <v>25784538829.65731</v>
       </c>
       <c r="M3" s="3">
-        <v>3326214883.838398</v>
+        <v>26331534604.66109</v>
       </c>
       <c r="N3" s="3">
-        <v>3391473925.195679</v>
+        <v>26886612327.6869</v>
       </c>
       <c r="O3" s="3">
-        <v>3457125457.577624</v>
+        <v>27440386767.30297</v>
       </c>
       <c r="P3" s="3">
-        <v>3535923246.01392</v>
+        <v>28059933837.37794</v>
       </c>
       <c r="Q3" s="3">
-        <v>3601921835.632152</v>
+        <v>28637527708.94907</v>
       </c>
       <c r="R3" s="3">
-        <v>41604572984.8067</v>
+        <v>330354430065.014</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -7086,46 +7086,46 @@
         <v>0</v>
       </c>
       <c r="E4" s="3">
-        <v>59013625754.90613</v>
+        <v>2824673820.668513</v>
       </c>
       <c r="F4" s="3">
-        <v>59291970846.39043</v>
+        <v>2892132503.559748</v>
       </c>
       <c r="G4" s="3">
-        <v>59597673202.9224</v>
+        <v>2945073514.468478</v>
       </c>
       <c r="H4" s="3">
-        <v>59979864661.2332</v>
+        <v>2997153077.667239</v>
       </c>
       <c r="I4" s="3">
-        <v>60521578337.89233</v>
+        <v>3062818764.410106</v>
       </c>
       <c r="J4" s="3">
-        <v>61237822832.92026</v>
+        <v>3128885547.708316</v>
       </c>
       <c r="K4" s="3">
-        <v>62127379495.47885</v>
+        <v>3181383526.957898</v>
       </c>
       <c r="L4" s="3">
-        <v>63153319620.30791</v>
+        <v>3259792881.108632</v>
       </c>
       <c r="M4" s="3">
-        <v>64286020237.35382</v>
+        <v>3326214883.838398</v>
       </c>
       <c r="N4" s="3">
-        <v>65527427133.00376</v>
+        <v>3391473925.195679</v>
       </c>
       <c r="O4" s="3">
-        <v>66848898017.66528</v>
+        <v>3457125457.577624</v>
       </c>
       <c r="P4" s="3">
-        <v>68222020110.84433</v>
+        <v>3535923246.01392</v>
       </c>
       <c r="Q4" s="3">
-        <v>69643822988.40005</v>
+        <v>3601921835.632152</v>
       </c>
       <c r="R4" s="3">
-        <v>819451423239.3188</v>
+        <v>41604572984.8067</v>
       </c>
     </row>
     <row r="5" spans="1:18">
@@ -7142,46 +7142,46 @@
         <v>0</v>
       </c>
       <c r="E5" s="3">
-        <v>550882261.7792752</v>
+        <v>59013625754.90613</v>
       </c>
       <c r="F5" s="3">
-        <v>553348887.0923566</v>
+        <v>59291970846.39043</v>
       </c>
       <c r="G5" s="3">
-        <v>558068640.1046562</v>
+        <v>59597673202.9224</v>
       </c>
       <c r="H5" s="3">
-        <v>564459006.9421008</v>
+        <v>59979864661.2332</v>
       </c>
       <c r="I5" s="3">
-        <v>572486986.0910172</v>
+        <v>60521578337.89233</v>
       </c>
       <c r="J5" s="3">
-        <v>581965641.6209706</v>
+        <v>61237822832.92026</v>
       </c>
       <c r="K5" s="3">
-        <v>592063097.9427336</v>
+        <v>62127379495.47885</v>
       </c>
       <c r="L5" s="3">
-        <v>603204835.1177481</v>
+        <v>63153319620.30791</v>
       </c>
       <c r="M5" s="3">
-        <v>615181350.4487659</v>
+        <v>64286020237.35382</v>
       </c>
       <c r="N5" s="3">
-        <v>627526131.6103884</v>
+        <v>65527427133.00376</v>
       </c>
       <c r="O5" s="3">
-        <v>640105159.1524134</v>
+        <v>66848898017.66528</v>
       </c>
       <c r="P5" s="3">
-        <v>653292232.6049073</v>
+        <v>68222020110.84433</v>
       </c>
       <c r="Q5" s="3">
-        <v>666750361.5668604</v>
+        <v>69643822988.40005</v>
       </c>
       <c r="R5" s="3">
-        <v>7779334592.074193</v>
+        <v>819451423239.3188</v>
       </c>
     </row>
     <row r="6" spans="1:18">
@@ -7198,46 +7198,46 @@
         <v>0</v>
       </c>
       <c r="E6" s="3">
-        <v>385800749.0446984</v>
+        <v>550882261.7792752</v>
       </c>
       <c r="F6" s="3">
-        <v>392905175.6015639</v>
+        <v>553348887.0923566</v>
       </c>
       <c r="G6" s="3">
-        <v>400080688.8739694</v>
+        <v>558068640.1046562</v>
       </c>
       <c r="H6" s="3">
-        <v>407201745.6201537</v>
+        <v>564459006.9421008</v>
       </c>
       <c r="I6" s="3">
-        <v>415943164.2399888</v>
+        <v>572486986.0910172</v>
       </c>
       <c r="J6" s="3">
-        <v>424845284.4305202</v>
+        <v>581965641.6209706</v>
       </c>
       <c r="K6" s="3">
-        <v>432134652.642395</v>
+        <v>592063097.9427336</v>
       </c>
       <c r="L6" s="3">
-        <v>442496837.8734584</v>
+        <v>603204835.1177481</v>
       </c>
       <c r="M6" s="3">
-        <v>451559207.5697356</v>
+        <v>615181350.4487659</v>
       </c>
       <c r="N6" s="3">
-        <v>460469579.4572726</v>
+        <v>627526131.6103884</v>
       </c>
       <c r="O6" s="3">
-        <v>469376006.5195322</v>
+        <v>640105159.1524134</v>
       </c>
       <c r="P6" s="3">
-        <v>479898292.2272025</v>
+        <v>653292232.6049073</v>
       </c>
       <c r="Q6" s="3">
-        <v>488964994.9722121</v>
+        <v>666750361.5668604</v>
       </c>
       <c r="R6" s="3">
-        <v>5651676379.072702</v>
+        <v>7779334592.074193</v>
       </c>
     </row>
     <row r="7" spans="1:18">
@@ -7254,46 +7254,46 @@
         <v>0</v>
       </c>
       <c r="E7" s="3">
-        <v>263348213.7307218</v>
+        <v>385800749.0446984</v>
       </c>
       <c r="F7" s="3">
-        <v>270966869.1744153</v>
+        <v>392905175.6015639</v>
       </c>
       <c r="G7" s="3">
-        <v>277692076.9216466</v>
+        <v>400080688.8739694</v>
       </c>
       <c r="H7" s="3">
-        <v>284045083.532236</v>
+        <v>407201745.6201537</v>
       </c>
       <c r="I7" s="3">
-        <v>291654961.317634</v>
+        <v>415943164.2399888</v>
       </c>
       <c r="J7" s="3">
-        <v>299614284.6548521</v>
+        <v>424845284.4305202</v>
       </c>
       <c r="K7" s="3">
-        <v>306300025.3087232</v>
+        <v>432134652.642395</v>
       </c>
       <c r="L7" s="3">
-        <v>315190797.047615</v>
+        <v>442496837.8734584</v>
       </c>
       <c r="M7" s="3">
-        <v>323469363.1907931</v>
+        <v>451559207.5697356</v>
       </c>
       <c r="N7" s="3">
-        <v>331410303.2703747</v>
+        <v>460469579.4572726</v>
       </c>
       <c r="O7" s="3">
-        <v>339355560.7691297</v>
+        <v>469376006.5195322</v>
       </c>
       <c r="P7" s="3">
-        <v>348595385.114009</v>
+        <v>479898292.2272025</v>
       </c>
       <c r="Q7" s="3">
-        <v>356835912.6742629</v>
+        <v>488964994.9722121</v>
       </c>
       <c r="R7" s="3">
-        <v>4008478836.706414</v>
+        <v>5651676379.072702</v>
       </c>
     </row>
     <row r="8" spans="1:18">
@@ -7310,46 +7310,46 @@
         <v>0</v>
       </c>
       <c r="E8" s="3">
-        <v>517454059.0277524</v>
+        <v>263348213.7307218</v>
       </c>
       <c r="F8" s="3">
-        <v>527607998.065537</v>
+        <v>270966869.1744153</v>
       </c>
       <c r="G8" s="3">
-        <v>540300421.8627679</v>
+        <v>277692076.9216466</v>
       </c>
       <c r="H8" s="3">
-        <v>550454360.9005525</v>
+        <v>284045083.532236</v>
       </c>
       <c r="I8" s="3">
-        <v>560608299.9383371</v>
+        <v>291654961.317634</v>
       </c>
       <c r="J8" s="3">
-        <v>573300723.7355678</v>
+        <v>299614284.6548521</v>
       </c>
       <c r="K8" s="3">
-        <v>585993147.5327988</v>
+        <v>306300025.3087232</v>
       </c>
       <c r="L8" s="3">
-        <v>596147086.5705835</v>
+        <v>315190797.047615</v>
       </c>
       <c r="M8" s="3">
-        <v>611377995.1272606</v>
+        <v>323469363.1907931</v>
       </c>
       <c r="N8" s="3">
-        <v>624070418.9244912</v>
+        <v>331410303.2703747</v>
       </c>
       <c r="O8" s="3">
-        <v>636762842.721722</v>
+        <v>339355560.7691297</v>
       </c>
       <c r="P8" s="3">
-        <v>649455266.5189528</v>
+        <v>348595385.114009</v>
       </c>
       <c r="Q8" s="3">
-        <v>664686175.0756301</v>
+        <v>356835912.6742629</v>
       </c>
       <c r="R8" s="3">
-        <v>7638218796.001953</v>
+        <v>4008478836.706414</v>
       </c>
     </row>
     <row r="9" spans="1:18">
@@ -7366,46 +7366,46 @@
         <v>0</v>
       </c>
       <c r="E9" s="3">
-        <v>85060.00982304836</v>
+        <v>517454059.0277524</v>
       </c>
       <c r="F9" s="3">
-        <v>87377.7511833305</v>
+        <v>527607998.065537</v>
       </c>
       <c r="G9" s="3">
-        <v>89380.97604674904</v>
+        <v>540300421.8627679</v>
       </c>
       <c r="H9" s="3">
-        <v>91301.05527788764</v>
+        <v>550454360.9005525</v>
       </c>
       <c r="I9" s="3">
-        <v>93622.74944426618</v>
+        <v>560608299.9383371</v>
       </c>
       <c r="J9" s="3">
-        <v>96023.98210304328</v>
+        <v>573300723.7355678</v>
       </c>
       <c r="K9" s="3">
-        <v>98019.82798761656</v>
+        <v>585993147.5327988</v>
       </c>
       <c r="L9" s="3">
-        <v>100751.5994268555</v>
+        <v>596147086.5705835</v>
       </c>
       <c r="M9" s="3">
-        <v>103225.6868523028</v>
+        <v>611377995.1272606</v>
       </c>
       <c r="N9" s="3">
-        <v>105625.6563460976</v>
+        <v>624070418.9244912</v>
       </c>
       <c r="O9" s="3">
-        <v>108025.3554714074</v>
+        <v>636762842.721722</v>
       </c>
       <c r="P9" s="3">
-        <v>110836.8324829971</v>
+        <v>649455266.5189528</v>
       </c>
       <c r="Q9" s="3">
-        <v>113303.816146075</v>
+        <v>664686175.0756301</v>
       </c>
       <c r="R9" s="3">
-        <v>1282555.298591677</v>
+        <v>7638218796.001953</v>
       </c>
     </row>
     <row r="10" spans="1:18">
@@ -7422,46 +7422,46 @@
         <v>0</v>
       </c>
       <c r="E10" s="3">
-        <v>85541470193.56918</v>
+        <v>85060.00982304836</v>
       </c>
       <c r="F10" s="3">
-        <v>86187427554.35443</v>
+        <v>87377.7511833305</v>
       </c>
       <c r="G10" s="3">
-        <v>86922452051.73706</v>
+        <v>89380.97604674904</v>
       </c>
       <c r="H10" s="3">
-        <v>87761170616.90669</v>
+        <v>91301.05527788764</v>
       </c>
       <c r="I10" s="3">
-        <v>88849114804.09862</v>
+        <v>93622.74944426618</v>
       </c>
       <c r="J10" s="3">
-        <v>90148703432.2594</v>
+        <v>96023.98210304328</v>
       </c>
       <c r="K10" s="3">
-        <v>91569937596.81255</v>
+        <v>98019.82798761656</v>
       </c>
       <c r="L10" s="3">
-        <v>93269797963.53577</v>
+        <v>100751.5994268555</v>
       </c>
       <c r="M10" s="3">
-        <v>95042342452.73726</v>
+        <v>103225.6868523028</v>
       </c>
       <c r="N10" s="3">
-        <v>96928156285.89066</v>
+        <v>105625.6563460976</v>
       </c>
       <c r="O10" s="3">
-        <v>98893365824.02509</v>
+        <v>108025.3554714074</v>
       </c>
       <c r="P10" s="3">
-        <v>100989432623.0793</v>
+        <v>110836.8324829971</v>
       </c>
       <c r="Q10" s="3">
-        <v>103082693291.142</v>
+        <v>113303.816146075</v>
       </c>
       <c r="R10" s="3">
-        <v>1205186064690.148</v>
+        <v>1282555.298591677</v>
       </c>
     </row>
     <row r="11" spans="1:18">
@@ -7478,46 +7478,46 @@
         <v>0</v>
       </c>
       <c r="E11" s="3">
-        <v>22719495997.45493</v>
+        <v>85194803013.39064</v>
       </c>
       <c r="F11" s="3">
-        <v>21589748846.89655</v>
+        <v>84404890393.58084</v>
       </c>
       <c r="G11" s="3">
-        <v>21951296446.34491</v>
+        <v>84929115541.41525</v>
       </c>
       <c r="H11" s="3">
-        <v>22348131950.14209</v>
+        <v>85583117736.72563</v>
       </c>
       <c r="I11" s="3">
-        <v>22807606219.78644</v>
+        <v>86522529344.67421</v>
       </c>
       <c r="J11" s="3">
-        <v>23299284255.63233</v>
+        <v>87714644472.82254</v>
       </c>
       <c r="K11" s="3">
-        <v>23763358443.0893</v>
+        <v>89069505812.59819</v>
       </c>
       <c r="L11" s="3">
-        <v>24335728575.61003</v>
+        <v>90712749984.36397</v>
       </c>
       <c r="M11" s="3">
-        <v>24877832515.91828</v>
+        <v>92444828225.81683</v>
       </c>
       <c r="N11" s="3">
-        <v>25439974138.43624</v>
+        <v>94310890727.90857</v>
       </c>
       <c r="O11" s="3">
-        <v>25994850413.06195</v>
+        <v>96258719122.24478</v>
       </c>
       <c r="P11" s="3">
-        <v>26610605289.7963</v>
+        <v>98337635291.84836</v>
       </c>
       <c r="Q11" s="3">
-        <v>27188818878.54765</v>
+        <v>100422892085.2535</v>
       </c>
       <c r="R11" s="3">
-        <v>312926731970.717</v>
+        <v>1175906321752.643</v>
       </c>
     </row>
     <row r="12" spans="1:18">
@@ -7534,46 +7534,46 @@
         <v>0</v>
       </c>
       <c r="E12" s="3">
-        <v>2717746279.21142</v>
+        <v>22719495997.45493</v>
       </c>
       <c r="F12" s="3">
-        <v>2894317790.600573</v>
+        <v>21589748846.89655</v>
       </c>
       <c r="G12" s="3">
-        <v>2947735736.458499</v>
+        <v>21951296446.34491</v>
       </c>
       <c r="H12" s="3">
-        <v>2999228863.59578</v>
+        <v>22348131950.14209</v>
       </c>
       <c r="I12" s="3">
-        <v>3064861924.15613</v>
+        <v>22807606219.78644</v>
       </c>
       <c r="J12" s="3">
-        <v>3131389146.821229</v>
+        <v>23299284255.63233</v>
       </c>
       <c r="K12" s="3">
-        <v>3183817120.098674</v>
+        <v>23763358443.0893</v>
       </c>
       <c r="L12" s="3">
-        <v>3261709964.96347</v>
+        <v>24335728575.61003</v>
       </c>
       <c r="M12" s="3">
-        <v>3329025840.756422</v>
+        <v>24877832515.91828</v>
       </c>
       <c r="N12" s="3">
-        <v>3393753743.501169</v>
+        <v>25439974138.43624</v>
       </c>
       <c r="O12" s="3">
-        <v>3459355425.14792</v>
+        <v>25994850413.06195</v>
       </c>
       <c r="P12" s="3">
-        <v>3538113632.307089</v>
+        <v>26610605289.7963</v>
       </c>
       <c r="Q12" s="3">
-        <v>3604485477.241018</v>
+        <v>27188818878.54765</v>
       </c>
       <c r="R12" s="3">
-        <v>41525540944.8594</v>
+        <v>312926731970.717</v>
       </c>
     </row>
     <row r="13" spans="1:18">
@@ -7590,46 +7590,46 @@
         <v>0</v>
       </c>
       <c r="E13" s="3">
-        <v>58905734197.09176</v>
+        <v>2717746279.21142</v>
       </c>
       <c r="F13" s="3">
-        <v>59056406256.72191</v>
+        <v>2894317790.600573</v>
       </c>
       <c r="G13" s="3">
-        <v>59147533631.09243</v>
+        <v>2947735736.458499</v>
       </c>
       <c r="H13" s="3">
-        <v>59336735606.577</v>
+        <v>2999228863.59578</v>
       </c>
       <c r="I13" s="3">
-        <v>59733848377.38585</v>
+        <v>3064861924.15613</v>
       </c>
       <c r="J13" s="3">
-        <v>60346106002.87461</v>
+        <v>3131389146.821229</v>
       </c>
       <c r="K13" s="3">
-        <v>61161592604.01636</v>
+        <v>3183817120.098674</v>
       </c>
       <c r="L13" s="3">
-        <v>62135251471.59244</v>
+        <v>3261709964.96347</v>
       </c>
       <c r="M13" s="3">
-        <v>63230910339.70621</v>
+        <v>3329025840.756422</v>
       </c>
       <c r="N13" s="3">
-        <v>64445881648.41473</v>
+        <v>3393753743.501169</v>
       </c>
       <c r="O13" s="3">
-        <v>65748804745.92617</v>
+        <v>3459355425.14792</v>
       </c>
       <c r="P13" s="3">
-        <v>67108842737.39155</v>
+        <v>3538113632.307089</v>
       </c>
       <c r="Q13" s="3">
-        <v>68521217410.90862</v>
+        <v>3604485477.241018</v>
       </c>
       <c r="R13" s="3">
-        <v>808878865029.6997</v>
+        <v>41525540944.8594</v>
       </c>
     </row>
     <row r="14" spans="1:18">
@@ -7646,46 +7646,46 @@
         <v>0</v>
       </c>
       <c r="E14" s="3">
-        <v>568131735.502313</v>
+        <v>58905734197.09176</v>
       </c>
       <c r="F14" s="3">
-        <v>571238500.3556887</v>
+        <v>59056406256.72191</v>
       </c>
       <c r="G14" s="3">
-        <v>576808941.2864491</v>
+        <v>59147533631.09243</v>
       </c>
       <c r="H14" s="3">
-        <v>583844477.0589781</v>
+        <v>59336735606.577</v>
       </c>
       <c r="I14" s="3">
-        <v>592351777.6998091</v>
+        <v>59733848377.38585</v>
       </c>
       <c r="J14" s="3">
-        <v>602186987.75893</v>
+        <v>60346106002.87461</v>
       </c>
       <c r="K14" s="3">
-        <v>612525816.6264801</v>
+        <v>61161592604.01636</v>
       </c>
       <c r="L14" s="3">
-        <v>623850089.6663957</v>
+        <v>62135251471.59244</v>
       </c>
       <c r="M14" s="3">
-        <v>635965134.8583637</v>
+        <v>63230910339.70621</v>
       </c>
       <c r="N14" s="3">
-        <v>648397591.4513019</v>
+        <v>64445881648.41473</v>
       </c>
       <c r="O14" s="3">
-        <v>661032895.3780229</v>
+        <v>65748804745.92617</v>
       </c>
       <c r="P14" s="3">
-        <v>674269156.7811122</v>
+        <v>67108842737.39155</v>
       </c>
       <c r="Q14" s="3">
-        <v>687759713.6863912</v>
+        <v>68521217410.90862</v>
       </c>
       <c r="R14" s="3">
-        <v>8038362818.110236</v>
+        <v>808878865029.6997</v>
       </c>
     </row>
     <row r="15" spans="1:18">
@@ -7702,46 +7702,46 @@
         <v>0</v>
       </c>
       <c r="E15" s="3">
-        <v>385906549.1300633</v>
+        <v>568131735.502313</v>
       </c>
       <c r="F15" s="3">
-        <v>394841285.339397</v>
+        <v>571238500.3556887</v>
       </c>
       <c r="G15" s="3">
-        <v>402178302.6803991</v>
+        <v>576808941.2864491</v>
       </c>
       <c r="H15" s="3">
-        <v>409300838.8005061</v>
+        <v>583844477.0589781</v>
       </c>
       <c r="I15" s="3">
-        <v>418049158.487105</v>
+        <v>592351777.6998091</v>
       </c>
       <c r="J15" s="3">
-        <v>426958490.3009185</v>
+        <v>602186987.75893</v>
       </c>
       <c r="K15" s="3">
-        <v>434239114.6789761</v>
+        <v>612525816.6264801</v>
       </c>
       <c r="L15" s="3">
-        <v>444606819.4734921</v>
+        <v>623850089.6663957</v>
       </c>
       <c r="M15" s="3">
-        <v>453675678.9584904</v>
+        <v>635965134.8583637</v>
       </c>
       <c r="N15" s="3">
-        <v>462577564.6360836</v>
+        <v>648397591.4513019</v>
       </c>
       <c r="O15" s="3">
-        <v>471481797.9816924</v>
+        <v>661032895.3780229</v>
       </c>
       <c r="P15" s="3">
-        <v>482009559.6614543</v>
+        <v>674269156.7811122</v>
       </c>
       <c r="Q15" s="3">
-        <v>491075211.3628312</v>
+        <v>687759713.6863912</v>
       </c>
       <c r="R15" s="3">
-        <v>5676900371.491409</v>
+        <v>8038362818.110236</v>
       </c>
     </row>
     <row r="16" spans="1:18">
@@ -7758,46 +7758,46 @@
         <v>0</v>
       </c>
       <c r="E16" s="3">
-        <v>172991699.2167722</v>
+        <v>385906549.1300633</v>
       </c>
       <c r="F16" s="3">
-        <v>181254460.1370325</v>
+        <v>394841285.339397</v>
       </c>
       <c r="G16" s="3">
-        <v>188458735.4417266</v>
+        <v>402178302.6803991</v>
       </c>
       <c r="H16" s="3">
-        <v>194861459.0214449</v>
+        <v>409300838.8005061</v>
       </c>
       <c r="I16" s="3">
-        <v>202137806.3348214</v>
+        <v>418049158.487105</v>
       </c>
       <c r="J16" s="3">
-        <v>210169337.7256945</v>
+        <v>426958490.3009185</v>
       </c>
       <c r="K16" s="3">
-        <v>217289197.7445626</v>
+        <v>434239114.6789761</v>
       </c>
       <c r="L16" s="3">
-        <v>225498446.4254824</v>
+        <v>444606819.4734921</v>
       </c>
       <c r="M16" s="3">
-        <v>234218341.9755156</v>
+        <v>453675678.9584904</v>
       </c>
       <c r="N16" s="3">
-        <v>242214607.3852603</v>
+        <v>462577564.6360836</v>
       </c>
       <c r="O16" s="3">
-        <v>250216046.1426421</v>
+        <v>471481797.9816924</v>
       </c>
       <c r="P16" s="3">
-        <v>259177474.5817247</v>
+        <v>482009559.6614543</v>
       </c>
       <c r="Q16" s="3">
-        <v>267815794.8797937</v>
+        <v>491075211.3628312</v>
       </c>
       <c r="R16" s="3">
-        <v>2846303407.012473</v>
+        <v>5676900371.491409</v>
       </c>
     </row>
     <row r="17" spans="1:18">
@@ -7814,46 +7814,46 @@
         <v>0</v>
       </c>
       <c r="E17" s="3">
-        <v>496545126.0286096</v>
+        <v>172991699.2167722</v>
       </c>
       <c r="F17" s="3">
-        <v>506699065.0663942</v>
+        <v>181254460.1370325</v>
       </c>
       <c r="G17" s="3">
-        <v>519391488.8636248</v>
+        <v>188458735.4417266</v>
       </c>
       <c r="H17" s="3">
-        <v>529545427.9014096</v>
+        <v>194861459.0214449</v>
       </c>
       <c r="I17" s="3">
-        <v>539699366.9391943</v>
+        <v>202137806.3348214</v>
       </c>
       <c r="J17" s="3">
-        <v>552391790.736425</v>
+        <v>210169337.7256945</v>
       </c>
       <c r="K17" s="3">
-        <v>565084214.533656</v>
+        <v>217289197.7445626</v>
       </c>
       <c r="L17" s="3">
-        <v>575238153.5714406</v>
+        <v>225498446.4254824</v>
       </c>
       <c r="M17" s="3">
-        <v>590469062.1281174</v>
+        <v>234218341.9755156</v>
       </c>
       <c r="N17" s="3">
-        <v>603161485.9253483</v>
+        <v>242214607.3852603</v>
       </c>
       <c r="O17" s="3">
-        <v>615853909.7225791</v>
+        <v>250216046.1426421</v>
       </c>
       <c r="P17" s="3">
-        <v>628546333.51981</v>
+        <v>259177474.5817247</v>
       </c>
       <c r="Q17" s="3">
-        <v>643777242.0764873</v>
+        <v>267815794.8797937</v>
       </c>
       <c r="R17" s="3">
-        <v>7366402667.013096</v>
+        <v>2846303407.012473</v>
       </c>
     </row>
     <row r="18" spans="1:18">
@@ -7870,46 +7870,46 @@
         <v>0</v>
       </c>
       <c r="E18" s="3">
-        <v>64528.01488962576</v>
+        <v>496545126.0286096</v>
       </c>
       <c r="F18" s="3">
-        <v>66759.14210145974</v>
+        <v>506699065.0663942</v>
       </c>
       <c r="G18" s="3">
-        <v>68864.60800164791</v>
+        <v>519391488.8636248</v>
       </c>
       <c r="H18" s="3">
-        <v>70791.22944198454</v>
+        <v>529545427.9014096</v>
       </c>
       <c r="I18" s="3">
-        <v>73030.85905438749</v>
+        <v>539699366.9391943</v>
       </c>
       <c r="J18" s="3">
-        <v>75441.57424663815</v>
+        <v>552391790.736425</v>
       </c>
       <c r="K18" s="3">
-        <v>77531.16812264835</v>
+        <v>565084214.533656</v>
       </c>
       <c r="L18" s="3">
-        <v>80102.00821263029</v>
+        <v>575238153.5714406</v>
       </c>
       <c r="M18" s="3">
-        <v>82669.43243499412</v>
+        <v>590469062.1281174</v>
       </c>
       <c r="N18" s="3">
-        <v>85077.43058664071</v>
+        <v>603161485.9253483</v>
       </c>
       <c r="O18" s="3">
-        <v>87484.8471815134</v>
+        <v>615853909.7225791</v>
       </c>
       <c r="P18" s="3">
-        <v>90227.13223671311</v>
+        <v>628546333.51981</v>
       </c>
       <c r="Q18" s="3">
-        <v>92779.27641959638</v>
+        <v>643777242.0764873</v>
       </c>
       <c r="R18" s="3">
-        <v>1015286.72293048</v>
+        <v>7366402667.013096</v>
       </c>
     </row>
     <row r="19" spans="1:18">
@@ -7926,46 +7926,46 @@
         <v>0</v>
       </c>
       <c r="E19" s="3">
-        <v>85194803013.39064</v>
+        <v>64528.01488962576</v>
       </c>
       <c r="F19" s="3">
-        <v>84404890393.58084</v>
+        <v>66759.14210145974</v>
       </c>
       <c r="G19" s="3">
-        <v>84929115541.41525</v>
+        <v>68864.60800164791</v>
       </c>
       <c r="H19" s="3">
-        <v>85583117736.72563</v>
+        <v>70791.22944198454</v>
       </c>
       <c r="I19" s="3">
-        <v>86522529344.67421</v>
+        <v>73030.85905438749</v>
       </c>
       <c r="J19" s="3">
-        <v>87714644472.82254</v>
+        <v>75441.57424663815</v>
       </c>
       <c r="K19" s="3">
-        <v>89069505812.59819</v>
+        <v>77531.16812264835</v>
       </c>
       <c r="L19" s="3">
-        <v>90712749984.36397</v>
+        <v>80102.00821263029</v>
       </c>
       <c r="M19" s="3">
-        <v>92444828225.81683</v>
+        <v>82669.43243499412</v>
       </c>
       <c r="N19" s="3">
-        <v>94310890727.90857</v>
+        <v>85077.43058664071</v>
       </c>
       <c r="O19" s="3">
-        <v>96258719122.24478</v>
+        <v>87484.8471815134</v>
       </c>
       <c r="P19" s="3">
-        <v>98337635291.84836</v>
+        <v>90227.13223671311</v>
       </c>
       <c r="Q19" s="3">
-        <v>100422892085.2535</v>
+        <v>92779.27641959638</v>
       </c>
       <c r="R19" s="3">
-        <v>1175906321752.643</v>
+        <v>1015286.72293048</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Changes to output file
</commit_message>
<xml_diff>
--- a/tests/optim_results_stillbirths.xlsx
+++ b/tests/optim_results_stillbirths.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="474" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="476" uniqueCount="70">
   <si>
     <t>Version</t>
   </si>
@@ -25,10 +25,10 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2.0.11</t>
+    <t>2.1.0</t>
   </si>
   <si>
-    <t>2025-06-30</t>
+    <t>2025-07-15</t>
   </si>
   <si>
     <t>Scenario</t>
@@ -609,7 +609,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R57"/>
+  <dimension ref="A1:R59"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
@@ -1616,8 +1616,8 @@
       <c r="Q18" s="3">
         <v>88.98045013788482</v>
       </c>
-      <c r="R18" s="3">
-        <v>1160.304421895408</v>
+      <c r="R18" s="3" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="19" spans="1:18">
@@ -2237,60 +2237,20 @@
       </c>
     </row>
     <row r="30" spans="1:18">
-      <c r="A30" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="B30" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C30" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D30" s="3">
-        <v>0</v>
-      </c>
-      <c r="E30" s="3">
-        <v>1175834.964281828</v>
-      </c>
-      <c r="F30" s="3">
-        <v>1182781.881046102</v>
-      </c>
-      <c r="G30" s="3">
-        <v>1192069.211077601</v>
-      </c>
-      <c r="H30" s="3">
-        <v>1203344.978747569</v>
-      </c>
-      <c r="I30" s="3">
-        <v>1217061.778131621</v>
-      </c>
-      <c r="J30" s="3">
-        <v>1233074.555447907</v>
-      </c>
-      <c r="K30" s="3">
-        <v>1251382.125139609</v>
-      </c>
-      <c r="L30" s="3">
-        <v>1271458.54185541</v>
-      </c>
-      <c r="M30" s="3">
-        <v>1292897.02791465</v>
-      </c>
-      <c r="N30" s="3">
-        <v>1315890.778520255</v>
-      </c>
-      <c r="O30" s="3">
-        <v>1340014.072920505</v>
-      </c>
-      <c r="P30" s="3">
-        <v>1364822.616915715</v>
-      </c>
-      <c r="Q30" s="3">
-        <v>1390322.477428165</v>
-      </c>
-      <c r="R30" s="3">
-        <v>16430955.00942694</v>
-      </c>
+      <c r="A30" s="2"/>
+      <c r="B30" s="3"/>
+      <c r="C30" s="3"/>
+      <c r="D30" s="3"/>
+      <c r="E30" s="3"/>
+      <c r="F30" s="3"/>
+      <c r="G30" s="3"/>
+      <c r="H30" s="3"/>
+      <c r="I30" s="3"/>
+      <c r="J30" s="3"/>
+      <c r="K30" s="3"/>
+      <c r="L30" s="3"/>
+      <c r="M30" s="3"/>
+      <c r="N30" s="3"/>
     </row>
     <row r="31" spans="1:18">
       <c r="A31" s="2" t="s">
@@ -2300,52 +2260,52 @@
         <v>9</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D31" s="3">
         <v>0</v>
       </c>
       <c r="E31" s="3">
-        <v>193680.9339243412</v>
+        <v>1175835.304263683</v>
       </c>
       <c r="F31" s="3">
-        <v>184049.9771793931</v>
+        <v>1182781.597952038</v>
       </c>
       <c r="G31" s="3">
-        <v>187132.1263928751</v>
+        <v>1192067.228493056</v>
       </c>
       <c r="H31" s="3">
-        <v>190515.1006894168</v>
+        <v>1203340.798545182</v>
       </c>
       <c r="I31" s="3">
-        <v>194432.0628292852</v>
+        <v>1217055.551833297</v>
       </c>
       <c r="J31" s="3">
-        <v>198623.5581504572</v>
+        <v>1233066.687326472</v>
       </c>
       <c r="K31" s="3">
-        <v>202579.7340289588</v>
+        <v>1251373.021872303</v>
       </c>
       <c r="L31" s="3">
-        <v>207459.1196381041</v>
+        <v>1271448.540818983</v>
       </c>
       <c r="M31" s="3">
-        <v>212080.4896480166</v>
+        <v>1292886.384538984</v>
       </c>
       <c r="N31" s="3">
-        <v>216872.6784562199</v>
+        <v>1315879.676270263</v>
       </c>
       <c r="O31" s="3">
-        <v>221602.931059271</v>
+        <v>1340002.647481795</v>
       </c>
       <c r="P31" s="3">
-        <v>226852.1663243374</v>
+        <v>1364810.967245214</v>
       </c>
       <c r="Q31" s="3">
-        <v>231781.3666855448</v>
+        <v>1390310.671271908</v>
       </c>
       <c r="R31" s="3">
-        <v>2667662.245006221</v>
+        <v>16430859.07791318</v>
       </c>
     </row>
     <row r="32" spans="1:18">
@@ -2356,52 +2316,52 @@
         <v>9</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D32" s="3">
         <v>0</v>
       </c>
       <c r="E32" s="3">
-        <v>760854.8538751315</v>
+        <v>193680.9928677323</v>
       </c>
       <c r="F32" s="3">
-        <v>762801.0068172098</v>
+        <v>184056.2172476264</v>
       </c>
       <c r="G32" s="3">
-        <v>763978.0519055324</v>
+        <v>187138.3531848086</v>
       </c>
       <c r="H32" s="3">
-        <v>766421.8758111735</v>
+        <v>190521.2857362549</v>
       </c>
       <c r="I32" s="3">
-        <v>771551.1757566555</v>
+        <v>194438.2604815272</v>
       </c>
       <c r="J32" s="3">
-        <v>779459.3903392383</v>
+        <v>198629.7699332653</v>
       </c>
       <c r="K32" s="3">
-        <v>789992.608322276</v>
+        <v>202585.9093473277</v>
       </c>
       <c r="L32" s="3">
-        <v>802568.8555333732</v>
+        <v>207465.3038237075</v>
       </c>
       <c r="M32" s="3">
-        <v>816720.9135521465</v>
+        <v>212086.6907215916</v>
       </c>
       <c r="N32" s="3">
-        <v>832414.0685590414</v>
+        <v>216878.8428937214</v>
       </c>
       <c r="O32" s="3">
-        <v>849243.2512605201</v>
+        <v>221609.0859182072</v>
       </c>
       <c r="P32" s="3">
-        <v>866810.1574601564</v>
+        <v>226858.3329249891</v>
       </c>
       <c r="Q32" s="3">
-        <v>885053.0694700507</v>
+        <v>231787.5261433228</v>
       </c>
       <c r="R32" s="3">
-        <v>10447869.27866251</v>
+        <v>2667736.571224082</v>
       </c>
     </row>
     <row r="33" spans="1:18">
@@ -2412,52 +2372,52 @@
         <v>9</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D33" s="3">
         <v>0</v>
       </c>
       <c r="E33" s="3">
-        <v>57321.78816640169</v>
+        <v>760854.516313656</v>
       </c>
       <c r="F33" s="3">
-        <v>57598.37311830824</v>
+        <v>762801.2709406794</v>
       </c>
       <c r="G33" s="3">
-        <v>57920.70975261508</v>
+        <v>763979.6181257832</v>
       </c>
       <c r="H33" s="3">
-        <v>58348.18023307858</v>
+        <v>766424.6744200211</v>
       </c>
       <c r="I33" s="3">
-        <v>58933.77618897777</v>
+        <v>771554.9143734995</v>
       </c>
       <c r="J33" s="3">
-        <v>59675.8045614947</v>
+        <v>779463.8088945907</v>
       </c>
       <c r="K33" s="3">
-        <v>60569.34109156278</v>
+        <v>789997.5106552148</v>
       </c>
       <c r="L33" s="3">
-        <v>61578.95543214476</v>
+        <v>802574.0968109665</v>
       </c>
       <c r="M33" s="3">
-        <v>62679.31139912491</v>
+        <v>816726.3927540452</v>
       </c>
       <c r="N33" s="3">
-        <v>63875.04688433809</v>
+        <v>832419.7151459286</v>
       </c>
       <c r="O33" s="3">
-        <v>65139.81841336723</v>
+        <v>849249.0125194135</v>
       </c>
       <c r="P33" s="3">
-        <v>66447.98072752243</v>
+        <v>866815.9972071933</v>
       </c>
       <c r="Q33" s="3">
-        <v>67798.75256951446</v>
+        <v>885058.9639740072</v>
       </c>
       <c r="R33" s="3">
-        <v>797887.8385384508</v>
+        <v>10447920.492135</v>
       </c>
     </row>
     <row r="34" spans="1:18">
@@ -2468,52 +2428,52 @@
         <v>9</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D34" s="3">
         <v>0</v>
       </c>
       <c r="E34" s="3">
-        <v>405972.8689105673</v>
+        <v>57321.75159615651</v>
       </c>
       <c r="F34" s="3">
-        <v>407837.2299962604</v>
+        <v>57598.33589730674</v>
       </c>
       <c r="G34" s="3">
-        <v>410030.9612581025</v>
+        <v>57920.65965833022</v>
       </c>
       <c r="H34" s="3">
-        <v>412907.1742424635</v>
+        <v>58348.10001597353</v>
       </c>
       <c r="I34" s="3">
-        <v>416858.1009372469</v>
+        <v>58933.6618961139</v>
       </c>
       <c r="J34" s="3">
-        <v>421872.9193536231</v>
+        <v>59675.66074533485</v>
       </c>
       <c r="K34" s="3">
-        <v>427919.113243547</v>
+        <v>60569.1742238659</v>
       </c>
       <c r="L34" s="3">
-        <v>434764.4032295443</v>
+        <v>61578.77138920808</v>
       </c>
       <c r="M34" s="3">
-        <v>442225.5874489979</v>
+        <v>62679.11490200154</v>
       </c>
       <c r="N34" s="3">
-        <v>450335.8863311257</v>
+        <v>63874.84137458662</v>
       </c>
       <c r="O34" s="3">
-        <v>458921.1247488323</v>
+        <v>65139.60641560221</v>
       </c>
       <c r="P34" s="3">
-        <v>467804.6661652726</v>
+        <v>66447.76415471175</v>
       </c>
       <c r="Q34" s="3">
-        <v>476974.8563706282</v>
+        <v>67798.53277177076</v>
       </c>
       <c r="R34" s="3">
-        <v>5634424.892236212</v>
+        <v>797885.9750409626</v>
       </c>
     </row>
     <row r="35" spans="1:18">
@@ -2524,52 +2484,52 @@
         <v>9</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D35" s="3">
         <v>0</v>
       </c>
       <c r="E35" s="3">
-        <v>1530716.949246393</v>
+        <v>405972.1131065895</v>
       </c>
       <c r="F35" s="3">
-        <v>1537745.657867051</v>
+        <v>407836.470374339</v>
       </c>
       <c r="G35" s="3">
-        <v>1546016.301725031</v>
+        <v>410030.1181374069</v>
       </c>
       <c r="H35" s="3">
-        <v>1556859.680316279</v>
+        <v>412906.1300310381</v>
       </c>
       <c r="I35" s="3">
-        <v>1571754.85295103</v>
+        <v>416856.8260824177</v>
       </c>
       <c r="J35" s="3">
-        <v>1590661.026433523</v>
+        <v>421871.4440251886</v>
       </c>
       <c r="K35" s="3">
-        <v>1613455.620218338</v>
+        <v>427917.481466108</v>
       </c>
       <c r="L35" s="3">
-        <v>1639262.994159239</v>
+        <v>434762.6548762303</v>
       </c>
       <c r="M35" s="3">
-        <v>1667392.354017799</v>
+        <v>442223.7549024466</v>
       </c>
       <c r="N35" s="3">
-        <v>1697968.960748171</v>
+        <v>450333.9931977502</v>
       </c>
       <c r="O35" s="3">
-        <v>1730336.199432193</v>
+        <v>458919.1881393528</v>
       </c>
       <c r="P35" s="3">
-        <v>1763828.108210599</v>
+        <v>467802.6990672618</v>
       </c>
       <c r="Q35" s="3">
-        <v>1798400.690527587</v>
+        <v>476972.868126953</v>
       </c>
       <c r="R35" s="3">
-        <v>21244399.39585323</v>
+        <v>5634405.741533083</v>
       </c>
     </row>
     <row r="36" spans="1:18">
@@ -2580,52 +2540,52 @@
         <v>9</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D36" s="3">
         <v>0</v>
       </c>
       <c r="E36" s="3">
-        <v>1879368.029990558</v>
+        <v>1530717.707470749</v>
       </c>
       <c r="F36" s="3">
-        <v>1887984.514745004</v>
+        <v>1537746.398518378</v>
       </c>
       <c r="G36" s="3">
-        <v>1898126.553230518</v>
+        <v>1546016.728481432</v>
       </c>
       <c r="H36" s="3">
-        <v>1911418.674325664</v>
+        <v>1556859.342934165</v>
       </c>
       <c r="I36" s="3">
-        <v>1929679.177699299</v>
+        <v>1571753.640124379</v>
       </c>
       <c r="J36" s="3">
-        <v>1952858.14122565</v>
+        <v>1590659.052195874</v>
       </c>
       <c r="K36" s="3">
-        <v>1980805.392370322</v>
+        <v>1613453.051061409</v>
       </c>
       <c r="L36" s="3">
-        <v>2012448.441956639</v>
+        <v>1639259.982753719</v>
       </c>
       <c r="M36" s="3">
-        <v>2046938.630067672</v>
+        <v>1667389.022390583</v>
       </c>
       <c r="N36" s="3">
-        <v>2084429.800194959</v>
+        <v>1697965.398218441</v>
       </c>
       <c r="O36" s="3">
-        <v>2124117.505767658</v>
+        <v>1730332.471861856</v>
       </c>
       <c r="P36" s="3">
-        <v>2165184.793648349</v>
+        <v>1763824.265385146</v>
       </c>
       <c r="Q36" s="3">
-        <v>2207576.794328701</v>
+        <v>1798396.767118962</v>
       </c>
       <c r="R36" s="3">
-        <v>26080936.449551</v>
+        <v>21244373.8285151</v>
       </c>
     </row>
     <row r="37" spans="1:18">
@@ -2636,52 +2596,52 @@
         <v>9</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D37" s="3">
         <v>0</v>
       </c>
       <c r="E37" s="3">
-        <v>901847.1917795757</v>
+        <v>1879368.068981183</v>
       </c>
       <c r="F37" s="3">
-        <v>907168.8404413904</v>
+        <v>1887984.532995411</v>
       </c>
       <c r="G37" s="3">
-        <v>914285.8875517375</v>
+        <v>1898126.186960509</v>
       </c>
       <c r="H37" s="3">
-        <v>922923.6940045216</v>
+        <v>1911417.372949229</v>
       </c>
       <c r="I37" s="3">
-        <v>933430.5613254531</v>
+        <v>1929676.804310683</v>
       </c>
       <c r="J37" s="3">
-        <v>945695.3295649479</v>
+        <v>1952854.835475728</v>
       </c>
       <c r="K37" s="3">
-        <v>959717.271801888</v>
+        <v>1980801.358303652</v>
       </c>
       <c r="L37" s="3">
-        <v>975094.3128428445</v>
+        <v>2012443.866240741</v>
       </c>
       <c r="M37" s="3">
-        <v>991514.213595163</v>
+        <v>2046933.662391028</v>
       </c>
       <c r="N37" s="3">
-        <v>1009125.190084892</v>
+        <v>2084424.550041605</v>
       </c>
       <c r="O37" s="3">
-        <v>1027601.591999935</v>
+        <v>2124112.053585607</v>
       </c>
       <c r="P37" s="3">
-        <v>1046603.002562976</v>
+        <v>2165179.200297696</v>
       </c>
       <c r="Q37" s="3">
-        <v>1066133.652218693</v>
+        <v>2207571.102474145</v>
       </c>
       <c r="R37" s="3">
-        <v>12601140.73977402</v>
+        <v>26080893.59500722</v>
       </c>
     </row>
     <row r="38" spans="1:18">
@@ -2692,52 +2652,52 @@
         <v>9</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D38" s="3">
-        <v>0.3411657413950535</v>
+        <v>0</v>
       </c>
       <c r="E38" s="3">
-        <v>0.338741145902639</v>
+        <v>901847.9157170992</v>
       </c>
       <c r="F38" s="3">
-        <v>0.336269503920948</v>
+        <v>907169.0867098067</v>
       </c>
       <c r="G38" s="3">
-        <v>0.3345627031832741</v>
+        <v>914284.8321422106</v>
       </c>
       <c r="H38" s="3">
-        <v>0.3334994452060328</v>
+        <v>922920.9542398655</v>
       </c>
       <c r="I38" s="3">
-        <v>0.3327842105587254</v>
+        <v>933426.2530787317</v>
       </c>
       <c r="J38" s="3">
-        <v>0.332453372548344</v>
+        <v>945689.7625073175</v>
       </c>
       <c r="K38" s="3">
-        <v>0.3325489652460839</v>
+        <v>959710.7575344221</v>
       </c>
       <c r="L38" s="3">
-        <v>0.3325837406374369</v>
+        <v>975087.1101287515</v>
       </c>
       <c r="M38" s="3">
-        <v>0.3328995671252145</v>
+        <v>991506.5181127666</v>
       </c>
       <c r="N38" s="3">
-        <v>0.3333429238303536</v>
+        <v>1009117.142429036</v>
       </c>
       <c r="O38" s="3">
-        <v>0.3338502604927557</v>
+        <v>1027593.296292328</v>
       </c>
       <c r="P38" s="3">
-        <v>0.3342814481122039</v>
+        <v>1046594.534722289</v>
       </c>
       <c r="Q38" s="3">
-        <v>0.3348691701940029</v>
-      </c>
-      <c r="R38" s="3" t="s">
-        <v>19</v>
+        <v>1066125.064077568</v>
+      </c>
+      <c r="R38" s="3">
+        <v>12601073.22769219</v>
       </c>
     </row>
     <row r="39" spans="1:18">
@@ -2748,49 +2708,49 @@
         <v>9</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D39" s="3">
-        <v>0.04535037632743646</v>
+        <v>0.3411657413950535</v>
       </c>
       <c r="E39" s="3">
-        <v>0.04487615002893723</v>
+        <v>0.3387427346297572</v>
       </c>
       <c r="F39" s="3">
-        <v>0.04498472597776491</v>
+        <v>0.3362722538854384</v>
       </c>
       <c r="G39" s="3">
-        <v>0.04510227809537754</v>
+        <v>0.3345661749514336</v>
       </c>
       <c r="H39" s="3">
-        <v>0.04520201485655706</v>
+        <v>0.3335033883629524</v>
       </c>
       <c r="I39" s="3">
-        <v>0.04530977398111725</v>
+        <v>0.3327884602730077</v>
       </c>
       <c r="J39" s="3">
-        <v>0.04540475739608452</v>
+        <v>0.332457803905315</v>
       </c>
       <c r="K39" s="3">
-        <v>0.04545423195937957</v>
+        <v>0.332553489432445</v>
       </c>
       <c r="L39" s="3">
-        <v>0.04553637761843177</v>
+        <v>0.3325883093906808</v>
       </c>
       <c r="M39" s="3">
-        <v>0.04559297497808926</v>
+        <v>0.3329041296060797</v>
       </c>
       <c r="N39" s="3">
-        <v>0.04563226821963461</v>
+        <v>0.3333474539669773</v>
       </c>
       <c r="O39" s="3">
-        <v>0.04566293962938627</v>
+        <v>0.3338547415576018</v>
       </c>
       <c r="P39" s="3">
-        <v>0.04571275123527276</v>
+        <v>0.3342858708887822</v>
       </c>
       <c r="Q39" s="3">
-        <v>0.04573839283201329</v>
+        <v>0.3348735211553743</v>
       </c>
       <c r="R39" s="3" t="s">
         <v>19</v>
@@ -2804,49 +2764,49 @@
         <v>9</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D40" s="3">
-        <v>0.2195512735036556</v>
+        <v>0.04535037632743646</v>
       </c>
       <c r="E40" s="3">
-        <v>0.2271854223126276</v>
+        <v>0.04487624322437406</v>
       </c>
       <c r="F40" s="3">
-        <v>0.2268126916927263</v>
+        <v>0.0449848017039336</v>
       </c>
       <c r="G40" s="3">
-        <v>0.2268178908171431</v>
+        <v>0.04510235069412313</v>
       </c>
       <c r="H40" s="3">
-        <v>0.2268815874361401</v>
+        <v>0.04520208957737901</v>
       </c>
       <c r="I40" s="3">
-        <v>0.2269083839406358</v>
+        <v>0.04530985176583999</v>
       </c>
       <c r="J40" s="3">
-        <v>0.2269611706797153</v>
+        <v>0.04540483702232926</v>
       </c>
       <c r="K40" s="3">
-        <v>0.2270455785877376</v>
+        <v>0.04545431227044335</v>
       </c>
       <c r="L40" s="3">
-        <v>0.227015914470804</v>
+        <v>0.04553645911671225</v>
       </c>
       <c r="M40" s="3">
-        <v>0.2270689119686186</v>
+        <v>0.04559305569838087</v>
       </c>
       <c r="N40" s="3">
-        <v>0.2270998554070574</v>
+        <v>0.04563234833484818</v>
       </c>
       <c r="O40" s="3">
-        <v>0.2271140794033218</v>
+        <v>0.04566301883441771</v>
       </c>
       <c r="P40" s="3">
-        <v>0.2270906108638255</v>
+        <v>0.04571282964407099</v>
       </c>
       <c r="Q40" s="3">
-        <v>0.2271268285391748</v>
+        <v>0.04573846960415755</v>
       </c>
       <c r="R40" s="3" t="s">
         <v>19</v>
@@ -2860,52 +2820,52 @@
         <v>9</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D41" s="3">
-        <v>0</v>
+        <v>0.2195512735036556</v>
       </c>
       <c r="E41" s="3">
-        <v>7402.80875685916</v>
+        <v>0.2271850070935322</v>
       </c>
       <c r="F41" s="3">
-        <v>7554.190101444537</v>
+        <v>0.2268122879880473</v>
       </c>
       <c r="G41" s="3">
-        <v>7743.416782176258</v>
+        <v>0.2268174640708815</v>
       </c>
       <c r="H41" s="3">
-        <v>7894.798126761633</v>
+        <v>0.2268811568233697</v>
       </c>
       <c r="I41" s="3">
-        <v>8046.179471347011</v>
+        <v>0.2269079588309105</v>
       </c>
       <c r="J41" s="3">
-        <v>8235.406152078733</v>
+        <v>0.2269607538969345</v>
       </c>
       <c r="K41" s="3">
-        <v>8424.632832810454</v>
+        <v>0.2270451707395189</v>
       </c>
       <c r="L41" s="3">
-        <v>8576.014177395828</v>
+        <v>0.2270155156007174</v>
       </c>
       <c r="M41" s="3">
-        <v>8803.086194273896</v>
+        <v>0.2270685217315657</v>
       </c>
       <c r="N41" s="3">
-        <v>8992.312875005615</v>
+        <v>0.2270994734759786</v>
       </c>
       <c r="O41" s="3">
-        <v>9181.539555737338</v>
+        <v>0.2271137056169461</v>
       </c>
       <c r="P41" s="3">
-        <v>9370.766236469059</v>
+        <v>0.2270902448521805</v>
       </c>
       <c r="Q41" s="3">
-        <v>9597.838253347125</v>
-      </c>
-      <c r="R41" s="3">
-        <v>109822.9895157067</v>
+        <v>0.2271264700070442</v>
+      </c>
+      <c r="R41" s="3" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="42" spans="1:18">
@@ -2916,52 +2876,52 @@
         <v>9</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D42" s="3">
         <v>0</v>
       </c>
       <c r="E42" s="3">
-        <v>358572.1515937085</v>
+        <v>7402.989558065228</v>
       </c>
       <c r="F42" s="3">
-        <v>370970.1788101819</v>
+        <v>7554.370902650606</v>
       </c>
       <c r="G42" s="3">
-        <v>382669.9256446229</v>
+        <v>7743.597583382327</v>
       </c>
       <c r="H42" s="3">
-        <v>393375.8616066968</v>
+        <v>7894.978927967704</v>
       </c>
       <c r="I42" s="3">
-        <v>405821.1353419254</v>
+        <v>8046.36027255308</v>
       </c>
       <c r="J42" s="3">
-        <v>419217.1050590093</v>
+        <v>8235.586953284801</v>
       </c>
       <c r="K42" s="3">
-        <v>430828.6535214814</v>
+        <v>8424.81363401652</v>
       </c>
       <c r="L42" s="3">
-        <v>445114.4124131034</v>
+        <v>8576.194978601898</v>
       </c>
       <c r="M42" s="3">
-        <v>459381.1898591706</v>
+        <v>8803.266995479964</v>
       </c>
       <c r="N42" s="3">
-        <v>472762.0614038244</v>
+        <v>8992.493676211685</v>
       </c>
       <c r="O42" s="3">
-        <v>486139.7013278551</v>
+        <v>9181.720356943406</v>
       </c>
       <c r="P42" s="3">
-        <v>501378.1532499879</v>
+        <v>9370.947037675129</v>
       </c>
       <c r="Q42" s="3">
-        <v>515560.02189106</v>
+        <v>9598.019054553193</v>
       </c>
       <c r="R42" s="3">
-        <v>5641790.551722628</v>
+        <v>109825.3399313855</v>
       </c>
     </row>
     <row r="43" spans="1:18">
@@ -2972,52 +2932,52 @@
         <v>9</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D43" s="3">
-        <v>0.18698022</v>
+        <v>0</v>
       </c>
       <c r="E43" s="3">
-        <v>0.1418464733936131</v>
+        <v>358638.3261512584</v>
       </c>
       <c r="F43" s="3">
-        <v>0.1434157221455479</v>
+        <v>371036.6325248702</v>
       </c>
       <c r="G43" s="3">
-        <v>0.1452970374106516</v>
+        <v>382736.0498367589</v>
       </c>
       <c r="H43" s="3">
-        <v>0.1467416187749276</v>
+        <v>393441.9647133123</v>
       </c>
       <c r="I43" s="3">
-        <v>0.1481355130737904</v>
+        <v>405887.5029423501</v>
       </c>
       <c r="J43" s="3">
-        <v>0.1498105791840118</v>
+        <v>419283.4420972573</v>
       </c>
       <c r="K43" s="3">
-        <v>0.1514152643652323</v>
+        <v>430894.6884102367</v>
       </c>
       <c r="L43" s="3">
-        <v>0.1526512698106022</v>
+        <v>445180.9659831104</v>
       </c>
       <c r="M43" s="3">
-        <v>0.1544305195847838</v>
+        <v>459447.4426049634</v>
       </c>
       <c r="N43" s="3">
-        <v>0.1558487621584068</v>
+        <v>472828.2882732772</v>
       </c>
       <c r="O43" s="3">
-        <v>0.1572120340896413</v>
+        <v>486205.9033239266</v>
       </c>
       <c r="P43" s="3">
-        <v>0.1585234705862281</v>
+        <v>501444.5782515256</v>
       </c>
       <c r="Q43" s="3">
-        <v>0.1600328413644559</v>
-      </c>
-      <c r="R43" s="3" t="s">
-        <v>19</v>
+        <v>515626.1724205</v>
+      </c>
+      <c r="R43" s="3">
+        <v>5642651.957533347</v>
       </c>
     </row>
     <row r="44" spans="1:18">
@@ -3028,52 +2988,52 @@
         <v>9</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D44" s="3">
-        <v>0</v>
+        <v>0.18698022</v>
       </c>
       <c r="E44" s="3">
-        <v>2134177.344298781</v>
+        <v>0.1418726511867717</v>
       </c>
       <c r="F44" s="3">
-        <v>2214969.379421716</v>
+        <v>0.1434414129099965</v>
       </c>
       <c r="G44" s="3">
-        <v>2299164.450020058</v>
+        <v>0.14532214429409</v>
       </c>
       <c r="H44" s="3">
-        <v>2385484.078891534</v>
+        <v>0.1467662773211617</v>
       </c>
       <c r="I44" s="3">
-        <v>2470725.421755608</v>
+        <v>0.1481597390139502</v>
       </c>
       <c r="J44" s="3">
-        <v>2557649.228635802</v>
+        <v>0.1498342852542112</v>
       </c>
       <c r="K44" s="3">
-        <v>2649521.287372913</v>
+        <v>0.1514384724087468</v>
       </c>
       <c r="L44" s="3">
-        <v>2740232.670360844</v>
+        <v>0.1526740942500916</v>
       </c>
       <c r="M44" s="3">
-        <v>2834805.988404087</v>
+        <v>0.154452791820092</v>
       </c>
       <c r="N44" s="3">
-        <v>2932460.168287891</v>
+        <v>0.1558705942309618</v>
       </c>
       <c r="O44" s="3">
-        <v>3032789.894420685</v>
+        <v>0.1572334430600149</v>
       </c>
       <c r="P44" s="3">
-        <v>3132856.792809556</v>
+        <v>0.1585444725419559</v>
       </c>
       <c r="Q44" s="3">
-        <v>3236624.754169994</v>
-      </c>
-      <c r="R44" s="3">
-        <v>34621461.45884947</v>
+        <v>0.1600533748750746</v>
+      </c>
+      <c r="R44" s="3" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="45" spans="1:18">
@@ -3084,52 +3044,52 @@
         <v>9</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D45" s="3">
-        <v>0.1886948075946863</v>
+        <v>0</v>
       </c>
       <c r="E45" s="3">
-        <v>0.1886169297295145</v>
+        <v>2134152.181190948</v>
       </c>
       <c r="F45" s="3">
-        <v>0.1886354567703546</v>
+        <v>2214944.246457329</v>
       </c>
       <c r="G45" s="3">
-        <v>0.1886415231009255</v>
+        <v>2299139.311079242</v>
       </c>
       <c r="H45" s="3">
-        <v>0.1886367497718057</v>
+        <v>2385458.95072664</v>
       </c>
       <c r="I45" s="3">
-        <v>0.1886246528752016</v>
+        <v>2470700.338314533</v>
       </c>
       <c r="J45" s="3">
-        <v>0.188608248191279</v>
+        <v>2557624.160387428</v>
       </c>
       <c r="K45" s="3">
-        <v>0.1885930736962086</v>
+        <v>2649496.203619596</v>
       </c>
       <c r="L45" s="3">
-        <v>0.1885867754428121</v>
+        <v>2740207.629595398</v>
       </c>
       <c r="M45" s="3">
-        <v>0.1885814245052841</v>
+        <v>2834780.941982774</v>
       </c>
       <c r="N45" s="3">
-        <v>0.1885801965413802</v>
+        <v>2932435.124326085</v>
       </c>
       <c r="O45" s="3">
-        <v>0.1885790703672576</v>
+        <v>3032764.856484</v>
       </c>
       <c r="P45" s="3">
-        <v>0.1885734633496969</v>
+        <v>3132831.78469258</v>
       </c>
       <c r="Q45" s="3">
-        <v>0.1885580263118771</v>
-      </c>
-      <c r="R45" s="3" t="s">
-        <v>19</v>
+        <v>3236599.743870288</v>
+      </c>
+      <c r="R45" s="3">
+        <v>34621135.47272684</v>
       </c>
     </row>
     <row r="46" spans="1:18">
@@ -3140,52 +3100,52 @@
         <v>9</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D46" s="3">
-        <v>0</v>
+        <v>0.1886948075946863</v>
       </c>
       <c r="E46" s="3">
-        <v>90.08415531364709</v>
+        <v>0.1886147058336633</v>
       </c>
       <c r="F46" s="3">
-        <v>86.83469220775501</v>
+        <v>0.1886333163487933</v>
       </c>
       <c r="G46" s="3">
-        <v>85.71518019675408</v>
+        <v>0.1886394605046268</v>
       </c>
       <c r="H46" s="3">
-        <v>85.16100768726336</v>
+        <v>0.188634762713751</v>
       </c>
       <c r="I46" s="3">
-        <v>84.80448223350994</v>
+        <v>0.1886227379091256</v>
       </c>
       <c r="J46" s="3">
-        <v>84.56802350263392</v>
+        <v>0.1886063995881327</v>
       </c>
       <c r="K46" s="3">
-        <v>84.43834332467047</v>
+        <v>0.1885912882332419</v>
       </c>
       <c r="L46" s="3">
-        <v>84.33293359485019</v>
+        <v>0.1885850521011188</v>
       </c>
       <c r="M46" s="3">
-        <v>84.27192301193948</v>
+        <v>0.1885797583278351</v>
       </c>
       <c r="N46" s="3">
-        <v>84.24865540216483</v>
+        <v>0.1885785860181443</v>
       </c>
       <c r="O46" s="3">
-        <v>84.24976018292675</v>
+        <v>0.1885775135067468</v>
       </c>
       <c r="P46" s="3">
-        <v>84.25738077899263</v>
+        <v>0.1885719580567511</v>
       </c>
       <c r="Q46" s="3">
-        <v>84.28632685643669</v>
-      </c>
-      <c r="R46" s="3">
-        <v>1107.252864293544</v>
+        <v>0.1885565692715625</v>
+      </c>
+      <c r="R46" s="3" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="47" spans="1:18">
@@ -3196,49 +3156,49 @@
         <v>9</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D47" s="3">
-        <v>0.01226890863757641</v>
+        <v>0</v>
       </c>
       <c r="E47" s="3">
-        <v>0.01204670666524164</v>
+        <v>90.08418272917784</v>
       </c>
       <c r="F47" s="3">
-        <v>0.01210585968202862</v>
+        <v>86.83614025640431</v>
       </c>
       <c r="G47" s="3">
-        <v>0.01214884491268141</v>
+        <v>85.7170809256703</v>
       </c>
       <c r="H47" s="3">
-        <v>0.01218127873614734</v>
+        <v>85.16311714052111</v>
       </c>
       <c r="I47" s="3">
-        <v>0.01221817083506928</v>
+        <v>84.80670620695976</v>
       </c>
       <c r="J47" s="3">
-        <v>0.01224863503809289</v>
+        <v>84.57031512895543</v>
       </c>
       <c r="K47" s="3">
-        <v>0.01226016132604589</v>
+        <v>84.44067429990889</v>
       </c>
       <c r="L47" s="3">
-        <v>0.01228962258358604</v>
+        <v>84.33528639730788</v>
       </c>
       <c r="M47" s="3">
-        <v>0.01230524718193481</v>
+        <v>84.2742876413061</v>
       </c>
       <c r="N47" s="3">
-        <v>0.01231536702077104</v>
+        <v>84.25102273156264</v>
       </c>
       <c r="O47" s="3">
-        <v>0.01232316701230193</v>
+        <v>84.25212479617734</v>
       </c>
       <c r="P47" s="3">
-        <v>0.01234011944019464</v>
+        <v>84.25973867453335</v>
       </c>
       <c r="Q47" s="3">
-        <v>0.01234498295397867</v>
+        <v>84.28867523614792</v>
       </c>
       <c r="R47" s="3" t="s">
         <v>19</v>
@@ -3252,49 +3212,49 @@
         <v>9</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D48" s="3">
-        <v>0.03308146768986005</v>
+        <v>0.01226890863757641</v>
       </c>
       <c r="E48" s="3">
-        <v>0.03282944336369559</v>
+        <v>0.0120467163087636</v>
       </c>
       <c r="F48" s="3">
-        <v>0.03287886629573628</v>
+        <v>0.01210586223910383</v>
       </c>
       <c r="G48" s="3">
-        <v>0.03295343318269613</v>
+        <v>0.01214884774408961</v>
       </c>
       <c r="H48" s="3">
-        <v>0.03302073612040972</v>
+        <v>0.0121812830176629</v>
       </c>
       <c r="I48" s="3">
-        <v>0.03309160314604797</v>
+        <v>0.0122181765188238</v>
       </c>
       <c r="J48" s="3">
-        <v>0.03315612235799163</v>
+        <v>0.01224864158671135</v>
       </c>
       <c r="K48" s="3">
-        <v>0.03319407063333369</v>
+        <v>0.01226016836272104</v>
       </c>
       <c r="L48" s="3">
-        <v>0.03324675503484573</v>
+        <v>0.01228963033417344</v>
       </c>
       <c r="M48" s="3">
-        <v>0.03328772779615446</v>
+        <v>0.01230525493118789</v>
       </c>
       <c r="N48" s="3">
-        <v>0.03331690119886357</v>
+        <v>0.01231537490481011</v>
       </c>
       <c r="O48" s="3">
-        <v>0.03333977261708435</v>
+        <v>0.01232317492459846</v>
       </c>
       <c r="P48" s="3">
-        <v>0.03337263179507812</v>
+        <v>0.01234012742657188</v>
       </c>
       <c r="Q48" s="3">
-        <v>0.03339340987803462</v>
+        <v>0.01234499070572747</v>
       </c>
       <c r="R48" s="3" t="s">
         <v>19</v>
@@ -3308,49 +3268,49 @@
         <v>9</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D49" s="3">
-        <v>121000.9090850509</v>
+        <v>0.03308146768986005</v>
       </c>
       <c r="E49" s="3">
-        <v>119045.9317004283</v>
+        <v>0.03282952691561045</v>
       </c>
       <c r="F49" s="3">
-        <v>120482.3383227453</v>
+        <v>0.03287893946482977</v>
       </c>
       <c r="G49" s="3">
-        <v>122086.4030456037</v>
+        <v>0.03295350295003352</v>
       </c>
       <c r="H49" s="3">
-        <v>123870.656513278</v>
+        <v>0.03302080655971611</v>
       </c>
       <c r="I49" s="3">
-        <v>126041.3310352337</v>
+        <v>0.03309167524701619</v>
       </c>
       <c r="J49" s="3">
-        <v>128423.6865773364</v>
+        <v>0.03315619543561791</v>
       </c>
       <c r="K49" s="3">
-        <v>130702.8832757888</v>
+        <v>0.03319414390772231</v>
       </c>
       <c r="L49" s="3">
-        <v>133456.6190459165</v>
+        <v>0.03324682878253881</v>
       </c>
       <c r="M49" s="3">
-        <v>136189.4934392393</v>
+        <v>0.03328780076719298</v>
       </c>
       <c r="N49" s="3">
-        <v>138947.1133353162</v>
+        <v>0.03331697343003807</v>
       </c>
       <c r="O49" s="3">
-        <v>141735.6117705673</v>
+        <v>0.03333984390981924</v>
       </c>
       <c r="P49" s="3">
-        <v>144787.5145756718</v>
+        <v>0.03337270221749911</v>
       </c>
       <c r="Q49" s="3">
-        <v>147719.0224676836</v>
+        <v>0.03339347889843008</v>
       </c>
       <c r="R49" s="3" t="s">
         <v>19</v>
@@ -3364,49 +3324,49 @@
         <v>9</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D50" s="3">
-        <v>326262.7331074112</v>
+        <v>121000.9090850509</v>
       </c>
       <c r="E50" s="3">
-        <v>324421.5851718169</v>
+        <v>119046.0262587818</v>
       </c>
       <c r="F50" s="3">
-        <v>327223.5757524818</v>
+        <v>120482.2877171642</v>
       </c>
       <c r="G50" s="3">
-        <v>331156.2666405824</v>
+        <v>122086.2845843769</v>
       </c>
       <c r="H50" s="3">
-        <v>335785.7865651741</v>
+        <v>123870.4942326121</v>
       </c>
       <c r="I50" s="3">
-        <v>341369.4048740941</v>
+        <v>126041.1378966607</v>
       </c>
       <c r="J50" s="3">
-        <v>347633.1405564931</v>
+        <v>128423.469005116</v>
       </c>
       <c r="K50" s="3">
-        <v>353874.6859896469</v>
+        <v>130702.6475838445</v>
       </c>
       <c r="L50" s="3">
-        <v>361036.2719457594</v>
+        <v>133456.3742510992</v>
       </c>
       <c r="M50" s="3">
-        <v>368415.0931122336</v>
+        <v>136189.2370665684</v>
       </c>
       <c r="N50" s="3">
-        <v>375895.1916781932</v>
+        <v>138946.8511378701</v>
       </c>
       <c r="O50" s="3">
-        <v>383459.3058307795</v>
+        <v>141735.3453567058</v>
       </c>
       <c r="P50" s="3">
-        <v>391563.5043790296</v>
+        <v>144787.2459696933</v>
       </c>
       <c r="Q50" s="3">
-        <v>399582.71975225</v>
+        <v>147718.7497117897</v>
       </c>
       <c r="R50" s="3" t="s">
         <v>19</v>
@@ -3420,52 +3380,52 @@
         <v>9</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D51" s="3">
-        <v>0</v>
+        <v>326262.7331074112</v>
       </c>
       <c r="E51" s="3">
-        <v>44246.0407564879</v>
+        <v>324422.4088199069</v>
       </c>
       <c r="F51" s="3">
-        <v>46359.40491265379</v>
+        <v>327224.0973997811</v>
       </c>
       <c r="G51" s="3">
-        <v>48202.04048531799</v>
+        <v>331156.5692447796</v>
       </c>
       <c r="H51" s="3">
-        <v>49839.66338712991</v>
+        <v>335785.9449271937</v>
       </c>
       <c r="I51" s="3">
-        <v>51700.73279822684</v>
+        <v>341369.4667624756</v>
       </c>
       <c r="J51" s="3">
-        <v>53754.95543935074</v>
+        <v>347633.1319444615</v>
       </c>
       <c r="K51" s="3">
-        <v>55576.00013688024</v>
+        <v>353874.6259154583</v>
       </c>
       <c r="L51" s="3">
-        <v>57675.67748186643</v>
+        <v>361036.1828644159</v>
       </c>
       <c r="M51" s="3">
-        <v>59905.96284033111</v>
+        <v>368414.9751841269</v>
       </c>
       <c r="N51" s="3">
-        <v>61951.16551087031</v>
+        <v>375895.0566531091</v>
       </c>
       <c r="O51" s="3">
-        <v>63997.69136715447</v>
+        <v>383459.1588296283</v>
       </c>
       <c r="P51" s="3">
-        <v>66289.75352821306</v>
+        <v>391563.3508154703</v>
       </c>
       <c r="Q51" s="3">
-        <v>68499.17440624617</v>
-      </c>
-      <c r="R51" s="3">
-        <v>727998.2630507289</v>
+        <v>399582.5569244476</v>
+      </c>
+      <c r="R51" s="3" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="52" spans="1:18">
@@ -3476,52 +3436,52 @@
         <v>9</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D52" s="3">
-        <v>0.5092287374537772</v>
+        <v>0</v>
       </c>
       <c r="E52" s="3">
-        <v>0.5124643392742281</v>
+        <v>44259.35931701703</v>
       </c>
       <c r="F52" s="3">
-        <v>0.5123975081964621</v>
+        <v>46372.72014859601</v>
       </c>
       <c r="G52" s="3">
-        <v>0.5123792321732593</v>
+        <v>48215.2819730656</v>
       </c>
       <c r="H52" s="3">
-        <v>0.5123877984182276</v>
+        <v>49852.8947654198</v>
       </c>
       <c r="I52" s="3">
-        <v>0.5124155264697793</v>
+        <v>51714.01140357759</v>
       </c>
       <c r="J52" s="3">
-        <v>0.5124229229444393</v>
+        <v>53768.22099416338</v>
       </c>
       <c r="K52" s="3">
-        <v>0.5124113506495643</v>
+        <v>55589.19872101418</v>
       </c>
       <c r="L52" s="3">
-        <v>0.512456891447295</v>
+        <v>57688.97477316566</v>
       </c>
       <c r="M52" s="3">
-        <v>0.5124451258294124</v>
+        <v>59919.19251129346</v>
       </c>
       <c r="N52" s="3">
-        <v>0.5124528422856667</v>
+        <v>61964.38436811615</v>
       </c>
       <c r="O52" s="3">
-        <v>0.5124595916881174</v>
+        <v>64010.89971082074</v>
       </c>
       <c r="P52" s="3">
-        <v>0.5124836796284932</v>
+        <v>66303.00101546283</v>
       </c>
       <c r="Q52" s="3">
-        <v>0.5124729733408402</v>
-      </c>
-      <c r="R52" s="3" t="s">
-        <v>19</v>
+        <v>68512.36083992774</v>
+      </c>
+      <c r="R52" s="3">
+        <v>728170.5005416402</v>
       </c>
     </row>
     <row r="53" spans="1:18">
@@ -3532,52 +3492,52 @@
         <v>9</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D53" s="3">
-        <v>0</v>
+        <v>0.5092287374537772</v>
       </c>
       <c r="E53" s="3">
-        <v>846408.8719133693</v>
+        <v>0.5124667228402195</v>
       </c>
       <c r="F53" s="3">
-        <v>866118.3812320065</v>
+        <v>0.5124000420338437</v>
       </c>
       <c r="G53" s="3">
-        <v>882244.2285624354</v>
+        <v>0.5123817506563494</v>
       </c>
       <c r="H53" s="3">
-        <v>897853.6717251246</v>
+        <v>0.5123902787310084</v>
       </c>
       <c r="I53" s="3">
-        <v>916994.6049238202</v>
+        <v>0.5124179652326236</v>
       </c>
       <c r="J53" s="3">
-        <v>936523.7864498167</v>
+        <v>0.5124253153636866</v>
       </c>
       <c r="K53" s="3">
-        <v>952515.1823746997</v>
+        <v>0.5124136945389287</v>
       </c>
       <c r="L53" s="3">
-        <v>975170.3530915184</v>
+        <v>0.512459191643642</v>
       </c>
       <c r="M53" s="3">
-        <v>995084.2189411632</v>
+        <v>0.5124473783784617</v>
       </c>
       <c r="N53" s="3">
-        <v>1014594.179839791</v>
+        <v>0.5124550478976651</v>
       </c>
       <c r="O53" s="3">
-        <v>1034110.653817215</v>
+        <v>0.5124617534574808</v>
       </c>
       <c r="P53" s="3">
-        <v>1057151.717499081</v>
+        <v>0.5124857996240592</v>
       </c>
       <c r="Q53" s="3">
-        <v>1077057.162663602</v>
-      </c>
-      <c r="R53" s="3">
-        <v>12451827.01303364</v>
+        <v>0.5124750497769561</v>
+      </c>
+      <c r="R53" s="3" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="54" spans="1:18">
@@ -3588,52 +3548,52 @@
         <v>9</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D54" s="3">
         <v>0</v>
       </c>
       <c r="E54" s="3">
-        <v>3028741.379624078</v>
+        <v>846408.842719867</v>
       </c>
       <c r="F54" s="3">
-        <v>3039763.659833033</v>
+        <v>866116.0383577015</v>
       </c>
       <c r="G54" s="3">
-        <v>3081052.927204179</v>
+        <v>882241.6896239708</v>
       </c>
       <c r="H54" s="3">
-        <v>3131912.708842842</v>
+        <v>897851.1340445473</v>
       </c>
       <c r="I54" s="3">
-        <v>3189861.716553305</v>
+        <v>916992.0610666556</v>
       </c>
       <c r="J54" s="3">
-        <v>3254517.590344205</v>
+        <v>936521.2356404738</v>
       </c>
       <c r="K54" s="3">
-        <v>3318037.287263173</v>
+        <v>952512.6444381119</v>
       </c>
       <c r="L54" s="3">
-        <v>3385139.7357473</v>
+        <v>975167.8109919636</v>
       </c>
       <c r="M54" s="3">
-        <v>3457285.954048042</v>
+        <v>995081.6702860963</v>
       </c>
       <c r="N54" s="3">
-        <v>3528137.293003849</v>
+        <v>1014591.644082182</v>
       </c>
       <c r="O54" s="3">
-        <v>3598007.922951123</v>
+        <v>1034108.122647971</v>
       </c>
       <c r="P54" s="3">
-        <v>3671585.443761185</v>
+        <v>1057149.181633392</v>
       </c>
       <c r="Q54" s="3">
-        <v>3746611.649127259</v>
+        <v>1077054.629649313</v>
       </c>
       <c r="R54" s="3">
-        <v>43430655.26830357</v>
+        <v>12451796.70518225</v>
       </c>
     </row>
     <row r="55" spans="1:18">
@@ -3644,52 +3604,52 @@
         <v>9</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D55" s="3">
-        <v>9862402</v>
+        <v>0</v>
       </c>
       <c r="E55" s="3">
-        <v>9882031.247918697</v>
+        <v>3028741.335417441</v>
       </c>
       <c r="F55" s="3">
-        <v>9952398.382875992</v>
+        <v>3039760.486168172</v>
       </c>
       <c r="G55" s="3">
-        <v>10049218.99349998</v>
+        <v>3081046.19781287</v>
       </c>
       <c r="H55" s="3">
-        <v>10168937.03825182</v>
+        <v>3131904.387059245</v>
       </c>
       <c r="I55" s="3">
-        <v>10315892.02153426</v>
+        <v>3189852.798170477</v>
       </c>
       <c r="J55" s="3">
-        <v>10484734.51759665</v>
+        <v>3254508.444208368</v>
       </c>
       <c r="K55" s="3">
-        <v>10660780.05010581</v>
+        <v>3318028.069447371</v>
       </c>
       <c r="L55" s="3">
-        <v>10859293.53307892</v>
+        <v>3385130.501558219</v>
       </c>
       <c r="M55" s="3">
-        <v>11067595.10196411</v>
+        <v>3457276.700986993</v>
       </c>
       <c r="N55" s="3">
-        <v>11282417.57642859</v>
+        <v>3528128.043765518</v>
       </c>
       <c r="O55" s="3">
-        <v>11501557.3211883</v>
+        <v>3597998.692643695</v>
       </c>
       <c r="P55" s="3">
-        <v>11733072.38048808</v>
+        <v>3671576.22013496</v>
       </c>
       <c r="Q55" s="3">
-        <v>11965915.46690432</v>
+        <v>3746602.426168614</v>
       </c>
       <c r="R55" s="3">
-        <v>149786245.6318356</v>
+        <v>43430554.30354194</v>
       </c>
     </row>
     <row r="56" spans="1:18">
@@ -3700,52 +3660,52 @@
         <v>9</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D56" s="3">
-        <v>2480858.588708919</v>
+        <v>9862402</v>
       </c>
       <c r="E56" s="3">
-        <v>2527889.0832816</v>
+        <v>9882031.186554927</v>
       </c>
       <c r="F56" s="3">
-        <v>2586677.201497451</v>
+        <v>9952392.100414585</v>
       </c>
       <c r="G56" s="3">
-        <v>2633707.696070131</v>
+        <v>10049206.90061093</v>
       </c>
       <c r="H56" s="3">
-        <v>2680738.190642813</v>
+        <v>10168920.14190948</v>
       </c>
       <c r="I56" s="3">
-        <v>2739526.308858664</v>
+        <v>10315871.41522115</v>
       </c>
       <c r="J56" s="3">
-        <v>2798314.427074515</v>
+        <v>10484711.14906682</v>
       </c>
       <c r="K56" s="3">
-        <v>2845344.921647196</v>
+        <v>10660754.70719197</v>
       </c>
       <c r="L56" s="3">
-        <v>2915890.663506217</v>
+        <v>10859266.76573832</v>
       </c>
       <c r="M56" s="3">
-        <v>2974678.781722068</v>
+        <v>11067567.2977237</v>
       </c>
       <c r="N56" s="3">
-        <v>3033466.899937919</v>
+        <v>11282389.06341378</v>
       </c>
       <c r="O56" s="3">
-        <v>3092255.018153772</v>
+        <v>11501528.31749437</v>
       </c>
       <c r="P56" s="3">
-        <v>3162800.760012793</v>
+        <v>11733043.02011698</v>
       </c>
       <c r="Q56" s="3">
-        <v>3221588.878228643</v>
+        <v>11965885.85872774</v>
       </c>
       <c r="R56" s="3">
-        <v>39693737.4193427</v>
+        <v>149785969.9241847</v>
       </c>
     </row>
     <row r="57" spans="1:18">
@@ -3756,53 +3716,125 @@
         <v>9</v>
       </c>
       <c r="C57" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D57" s="3">
+        <v>2480858.588708919</v>
+      </c>
+      <c r="E57" s="3">
+        <v>2527889.0832816</v>
+      </c>
+      <c r="F57" s="3">
+        <v>2586677.201497451</v>
+      </c>
+      <c r="G57" s="3">
+        <v>2633707.696070131</v>
+      </c>
+      <c r="H57" s="3">
+        <v>2680738.190642813</v>
+      </c>
+      <c r="I57" s="3">
+        <v>2739526.308858664</v>
+      </c>
+      <c r="J57" s="3">
+        <v>2798314.427074515</v>
+      </c>
+      <c r="K57" s="3">
+        <v>2845344.921647196</v>
+      </c>
+      <c r="L57" s="3">
+        <v>2915890.663506217</v>
+      </c>
+      <c r="M57" s="3">
+        <v>2974678.781722068</v>
+      </c>
+      <c r="N57" s="3">
+        <v>3033466.899937919</v>
+      </c>
+      <c r="O57" s="3">
+        <v>3092255.018153772</v>
+      </c>
+      <c r="P57" s="3">
+        <v>3162800.760012793</v>
+      </c>
+      <c r="Q57" s="3">
+        <v>3221588.878228643</v>
+      </c>
+      <c r="R57" s="3">
+        <v>39693737.4193427</v>
+      </c>
+    </row>
+    <row r="58" spans="1:18">
+      <c r="A58" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B58" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C58" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D57" s="3">
-        <v>0</v>
-      </c>
-      <c r="E57" s="3">
-        <v>46336.91148659605</v>
-      </c>
-      <c r="F57" s="3">
-        <v>49347.41270846425</v>
-      </c>
-      <c r="G57" s="3">
-        <v>50258.17566229402</v>
-      </c>
-      <c r="H57" s="3">
-        <v>51136.12092619868</v>
-      </c>
-      <c r="I57" s="3">
-        <v>52255.14860771639</v>
-      </c>
-      <c r="J57" s="3">
-        <v>53389.4215351275</v>
-      </c>
-      <c r="K57" s="3">
-        <v>54283.30569781082</v>
-      </c>
-      <c r="L57" s="3">
-        <v>55611.3597128407</v>
-      </c>
-      <c r="M57" s="3">
-        <v>56759.07898381168</v>
-      </c>
-      <c r="N57" s="3">
-        <v>57862.67394524668</v>
-      </c>
-      <c r="O57" s="3">
-        <v>58981.16662393755</v>
-      </c>
-      <c r="P57" s="3">
-        <v>60323.97485511514</v>
-      </c>
-      <c r="Q57" s="3">
-        <v>61455.59863009017</v>
-      </c>
-      <c r="R57" s="3">
-        <v>708000.3493752496</v>
-      </c>
+      <c r="D58" s="3">
+        <v>0</v>
+      </c>
+      <c r="E58" s="3">
+        <v>46337.96888682542</v>
+      </c>
+      <c r="F58" s="3">
+        <v>49347.39024856551</v>
+      </c>
+      <c r="G58" s="3">
+        <v>50258.14832120934</v>
+      </c>
+      <c r="H58" s="3">
+        <v>51136.09962706856</v>
+      </c>
+      <c r="I58" s="3">
+        <v>52255.12765785637</v>
+      </c>
+      <c r="J58" s="3">
+        <v>53389.39588118303</v>
+      </c>
+      <c r="K58" s="3">
+        <v>54283.28078113063</v>
+      </c>
+      <c r="L58" s="3">
+        <v>55611.34009950649</v>
+      </c>
+      <c r="M58" s="3">
+        <v>56759.0502423184</v>
+      </c>
+      <c r="N58" s="3">
+        <v>57862.65065421472</v>
+      </c>
+      <c r="O58" s="3">
+        <v>58981.14385748453</v>
+      </c>
+      <c r="P58" s="3">
+        <v>60323.95250716664</v>
+      </c>
+      <c r="Q58" s="3">
+        <v>61455.57249009677</v>
+      </c>
+      <c r="R58" s="3">
+        <v>708001.1212546265</v>
+      </c>
+    </row>
+    <row r="59" spans="1:18">
+      <c r="A59" s="2"/>
+      <c r="B59" s="3"/>
+      <c r="C59" s="3"/>
+      <c r="D59" s="3"/>
+      <c r="E59" s="3"/>
+      <c r="F59" s="3"/>
+      <c r="G59" s="3"/>
+      <c r="H59" s="3"/>
+      <c r="I59" s="3"/>
+      <c r="J59" s="3"/>
+      <c r="K59" s="3"/>
+      <c r="L59" s="3"/>
+      <c r="M59" s="3"/>
+      <c r="N59" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3811,7 +3843,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R55"/>
+  <dimension ref="A1:R57"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
@@ -5327,67 +5359,27 @@
       </c>
     </row>
     <row r="28" spans="1:18">
-      <c r="A28" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="B28" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="C28" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="D28" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="E28" s="3">
-        <v>0</v>
-      </c>
-      <c r="F28" s="3">
-        <v>0.002567075062468163</v>
-      </c>
-      <c r="G28" s="3">
-        <v>0.00247159469082187</v>
-      </c>
-      <c r="H28" s="3">
-        <v>0.002382510862562126</v>
-      </c>
-      <c r="I28" s="3">
-        <v>0.00229551812525578</v>
-      </c>
-      <c r="J28" s="3">
-        <v>0.002212053284320068</v>
-      </c>
-      <c r="K28" s="3">
-        <v>0.002134918052395384</v>
-      </c>
-      <c r="L28" s="3">
-        <v>0.002061310612330866</v>
-      </c>
-      <c r="M28" s="3">
-        <v>0.001988829505289415</v>
-      </c>
-      <c r="N28" s="3">
-        <v>0.001922372025891526</v>
-      </c>
-      <c r="O28" s="3">
-        <v>0.001857658711739989</v>
-      </c>
-      <c r="P28" s="3">
-        <v>0.001795383293092765</v>
-      </c>
-      <c r="Q28" s="3">
-        <v>0.001735614763602078</v>
-      </c>
-      <c r="R28" s="3">
-        <v>0.001679713402650515</v>
-      </c>
+      <c r="A28" s="2"/>
+      <c r="B28" s="3"/>
+      <c r="C28" s="3"/>
+      <c r="D28" s="3"/>
+      <c r="E28" s="3"/>
+      <c r="F28" s="3"/>
+      <c r="G28" s="3"/>
+      <c r="H28" s="3"/>
+      <c r="I28" s="3"/>
+      <c r="J28" s="3"/>
+      <c r="K28" s="3"/>
+      <c r="L28" s="3"/>
+      <c r="M28" s="3"/>
+      <c r="N28" s="3"/>
     </row>
     <row r="29" spans="1:18">
       <c r="A29" s="2" t="s">
         <v>39</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C29" s="3" t="s">
         <v>44</v>
@@ -5399,43 +5391,43 @@
         <v>0</v>
       </c>
       <c r="F29" s="3">
-        <v>0.002456508159028523</v>
+        <v>0.002626876079961963</v>
       </c>
       <c r="G29" s="3">
-        <v>0.002365140237846398</v>
+        <v>0.002529171455718381</v>
       </c>
       <c r="H29" s="3">
-        <v>0.002279893353500463</v>
+        <v>0.002438012384841051</v>
       </c>
       <c r="I29" s="3">
-        <v>0.002196647494392704</v>
+        <v>0.002348993117698648</v>
       </c>
       <c r="J29" s="3">
-        <v>0.002116777581062837</v>
+        <v>0.002263583930652497</v>
       </c>
       <c r="K29" s="3">
-        <v>0.002042964653134909</v>
+        <v>0.002184651803334625</v>
       </c>
       <c r="L29" s="3">
-        <v>0.001972527570975791</v>
+        <v>0.002109329649167925</v>
       </c>
       <c r="M29" s="3">
-        <v>0.00190316830936871</v>
+        <v>0.002035160066392544</v>
       </c>
       <c r="N29" s="3">
-        <v>0.001839573230768858</v>
+        <v>0.001967154434022359</v>
       </c>
       <c r="O29" s="3">
-        <v>0.001777647194193136</v>
+        <v>0.001900933597910035</v>
       </c>
       <c r="P29" s="3">
-        <v>0.001718054050131841</v>
+        <v>0.001837207449031194</v>
       </c>
       <c r="Q29" s="3">
-        <v>0.00166085982060049</v>
+        <v>0.001776046588272165</v>
       </c>
       <c r="R29" s="3">
-        <v>0.001607366196169313</v>
+        <v>0.001718842983255726</v>
       </c>
     </row>
     <row r="30" spans="1:18">
@@ -5443,7 +5435,7 @@
         <v>39</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C30" s="3" t="s">
         <v>44</v>
@@ -5455,43 +5447,43 @@
         <v>0</v>
       </c>
       <c r="F30" s="3">
-        <v>0.001410635896770717</v>
+        <v>0.002513733477266973</v>
       </c>
       <c r="G30" s="3">
-        <v>0.00140757968448265</v>
+        <v>0.002420237104629388</v>
       </c>
       <c r="H30" s="3">
-        <v>0.001394087341469662</v>
+        <v>0.002333004360774864</v>
       </c>
       <c r="I30" s="3">
-        <v>0.001373293890279159</v>
+        <v>0.002247819256823987</v>
       </c>
       <c r="J30" s="3">
-        <v>0.001350475038145597</v>
+        <v>0.002166088742628139</v>
       </c>
       <c r="K30" s="3">
-        <v>0.001324740749392845</v>
+        <v>0.00209055631367789</v>
       </c>
       <c r="L30" s="3">
-        <v>0.00129799651992155</v>
+        <v>0.002018478372143839</v>
       </c>
       <c r="M30" s="3">
-        <v>0.001274132780923575</v>
+        <v>0.00194750335941309</v>
       </c>
       <c r="N30" s="3">
-        <v>0.00124743734540452</v>
+        <v>0.001882426808586939</v>
       </c>
       <c r="O30" s="3">
-        <v>0.001221760007576078</v>
+        <v>0.001819058180771588</v>
       </c>
       <c r="P30" s="3">
-        <v>0.001197546561357245</v>
+        <v>0.00175807679111412</v>
       </c>
       <c r="Q30" s="3">
-        <v>0.001174492135394355</v>
+        <v>0.00169955019963872</v>
       </c>
       <c r="R30" s="3">
-        <v>0.001150272551926583</v>
+        <v>0.00164481042030651</v>
       </c>
     </row>
     <row r="31" spans="1:18">
@@ -5499,7 +5491,7 @@
         <v>39</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C31" s="3" t="s">
         <v>44</v>
@@ -5511,43 +5503,43 @@
         <v>0</v>
       </c>
       <c r="F31" s="3">
-        <v>0.0002503211431552996</v>
+        <v>0.001443497211647526</v>
       </c>
       <c r="G31" s="3">
-        <v>0.0002472315945356059</v>
+        <v>0.001440369829521683</v>
       </c>
       <c r="H31" s="3">
-        <v>0.0002460637264003582</v>
+        <v>0.001426565213675929</v>
       </c>
       <c r="I31" s="3">
-        <v>0.0002426655222415408</v>
+        <v>0.001405288504253844</v>
       </c>
       <c r="J31" s="3">
-        <v>0.0002386994563320606</v>
+        <v>0.001381938452249662</v>
       </c>
       <c r="K31" s="3">
-        <v>0.0002343160453360894</v>
+        <v>0.001355604713316605</v>
       </c>
       <c r="L31" s="3">
-        <v>0.0002296418715957639</v>
+        <v>0.001328237388064702</v>
       </c>
       <c r="M31" s="3">
-        <v>0.0002252826531286139</v>
+        <v>0.001303817619599434</v>
       </c>
       <c r="N31" s="3">
-        <v>0.0002207649588380092</v>
+        <v>0.001276500167421185</v>
       </c>
       <c r="O31" s="3">
-        <v>0.0002161682355905269</v>
+        <v>0.001250224539167385</v>
       </c>
       <c r="P31" s="3">
-        <v>0.0002118408792531711</v>
+        <v>0.001225446902309694</v>
       </c>
       <c r="Q31" s="3">
-        <v>0.000207736076208027</v>
+        <v>0.001201855293337325</v>
       </c>
       <c r="R31" s="3">
-        <v>0.0002035479011875169</v>
+        <v>0.001177071386615135</v>
       </c>
     </row>
     <row r="32" spans="1:18">
@@ -5555,7 +5547,7 @@
         <v>39</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C32" s="3" t="s">
         <v>44</v>
@@ -5564,46 +5556,46 @@
         <v>45</v>
       </c>
       <c r="E32" s="3">
-        <v>0.3538</v>
+        <v>0</v>
       </c>
       <c r="F32" s="3">
-        <v>0.7610161611665138</v>
+        <v>0.000256152472078929</v>
       </c>
       <c r="G32" s="3">
-        <v>0.7468577209587648</v>
+        <v>0.0002529909553379114</v>
       </c>
       <c r="H32" s="3">
-        <v>0.7298836818460656</v>
+        <v>0.0002517961699818421</v>
       </c>
       <c r="I32" s="3">
-        <v>0.7168500446702432</v>
+        <v>0.0002483190669875678</v>
       </c>
       <c r="J32" s="3">
-        <v>0.7042737280970808</v>
+        <v>0.0002442607064850759</v>
       </c>
       <c r="K32" s="3">
-        <v>0.6891605579662421</v>
+        <v>0.0002397751996773829</v>
       </c>
       <c r="L32" s="3">
-        <v>0.6746823949837581</v>
+        <v>0.0002349921279446757</v>
       </c>
       <c r="M32" s="3">
-        <v>0.6635306198600597</v>
+        <v>0.0002305313393253143</v>
       </c>
       <c r="N32" s="3">
-        <v>0.647477459702155</v>
+        <v>0.000225908379265602</v>
       </c>
       <c r="O32" s="3">
-        <v>0.6346814624748397</v>
+        <v>0.0002212045494584475</v>
       </c>
       <c r="P32" s="3">
-        <v>0.6223814341323041</v>
+        <v>0.0002167763618515439</v>
       </c>
       <c r="Q32" s="3">
-        <v>0.6105490874757962</v>
+        <v>0.0002125759129584818</v>
       </c>
       <c r="R32" s="3">
-        <v>0.5969308922161131</v>
+        <v>0.0002082901507778751</v>
       </c>
     </row>
     <row r="33" spans="1:18">
@@ -5611,7 +5603,7 @@
         <v>39</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C33" s="3" t="s">
         <v>44</v>
@@ -5620,46 +5612,46 @@
         <v>45</v>
       </c>
       <c r="E33" s="3">
-        <v>0.1</v>
+        <v>0.3538</v>
       </c>
       <c r="F33" s="3">
-        <v>0.0002579509746879906</v>
+        <v>0.7607799738069581</v>
       </c>
       <c r="G33" s="3">
-        <v>0.0002565457233052462</v>
+        <v>0.7466259277826426</v>
       </c>
       <c r="H33" s="3">
-        <v>0.0002552347144710252</v>
+        <v>0.7296571566966734</v>
       </c>
       <c r="I33" s="3">
-        <v>0.0002530333461828454</v>
+        <v>0.7166275646128044</v>
       </c>
       <c r="J33" s="3">
-        <v>0.0002502253053421964</v>
+        <v>0.7040551511985444</v>
       </c>
       <c r="K33" s="3">
-        <v>0.0002468664592081082</v>
+        <v>0.6889466715590907</v>
       </c>
       <c r="L33" s="3">
-        <v>0.0002430343182772099</v>
+        <v>0.6744730019885218</v>
       </c>
       <c r="M33" s="3">
-        <v>0.0002390255039053128</v>
+        <v>0.6633246879060668</v>
       </c>
       <c r="N33" s="3">
-        <v>0.0002348094471138756</v>
+        <v>0.6472765099728555</v>
       </c>
       <c r="O33" s="3">
-        <v>0.0002304212327731392</v>
+        <v>0.6344844840840639</v>
       </c>
       <c r="P33" s="3">
-        <v>0.0002260396596196866</v>
+        <v>0.6221882731522023</v>
       </c>
       <c r="Q33" s="3">
-        <v>0.000221728426471891</v>
+        <v>0.6103595987576734</v>
       </c>
       <c r="R33" s="3">
-        <v>0.0002174134926176375</v>
+        <v>0.5967456300121492</v>
       </c>
     </row>
     <row r="34" spans="1:18">
@@ -5667,7 +5659,7 @@
         <v>39</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C34" s="3" t="s">
         <v>44</v>
@@ -5676,46 +5668,46 @@
         <v>45</v>
       </c>
       <c r="E34" s="3">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="F34" s="3">
-        <v>0.0002607511907867704</v>
+        <v>0.0002639600435209947</v>
       </c>
       <c r="G34" s="3">
-        <v>0.0002575329109745895</v>
+        <v>0.0002625220573844941</v>
       </c>
       <c r="H34" s="3">
-        <v>0.0002563163816670398</v>
+        <v>0.0002611806214514344</v>
       </c>
       <c r="I34" s="3">
-        <v>0.0002527765856682716</v>
+        <v>0.0002589281325250978</v>
       </c>
       <c r="J34" s="3">
-        <v>0.0002486452670125631</v>
+        <v>0.0002560548067764714</v>
       </c>
       <c r="K34" s="3">
-        <v>0.0002440792138917597</v>
+        <v>0.0002526178058683669</v>
       </c>
       <c r="L34" s="3">
-        <v>0.000239210282912254</v>
+        <v>0.0002486964517393062</v>
       </c>
       <c r="M34" s="3">
-        <v>0.0002346694303423061</v>
+        <v>0.0002445942834943027</v>
       </c>
       <c r="N34" s="3">
-        <v>0.0002299634987895928</v>
+        <v>0.0002402800267475754</v>
       </c>
       <c r="O34" s="3">
-        <v>0.0002251752454067988</v>
+        <v>0.0002357895895965128</v>
       </c>
       <c r="P34" s="3">
-        <v>0.0002206675825553865</v>
+        <v>0.0002313059398437843</v>
       </c>
       <c r="Q34" s="3">
-        <v>0.0002163917460500281</v>
+        <v>0.0002268942632055325</v>
       </c>
       <c r="R34" s="3">
-        <v>0.0002120290637369967</v>
+        <v>0.0002224787961709672</v>
       </c>
     </row>
     <row r="35" spans="1:18">
@@ -5723,7 +5715,7 @@
         <v>39</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C35" s="3" t="s">
         <v>44</v>
@@ -5735,43 +5727,43 @@
         <v>0</v>
       </c>
       <c r="F35" s="3">
-        <v>0.001454378057460736</v>
+        <v>0.0002668254917488844</v>
       </c>
       <c r="G35" s="3">
-        <v>0.001451935436480021</v>
+        <v>0.0002635322451436578</v>
       </c>
       <c r="H35" s="3">
-        <v>0.001442096336695622</v>
+        <v>0.000262287677064419</v>
       </c>
       <c r="I35" s="3">
-        <v>0.001428426684495988</v>
+        <v>0.0002586656947787164</v>
       </c>
       <c r="J35" s="3">
-        <v>0.001411766891291532</v>
+        <v>0.0002544382359219541</v>
       </c>
       <c r="K35" s="3">
-        <v>0.001391850937163765</v>
+        <v>0.0002497658329972739</v>
       </c>
       <c r="L35" s="3">
-        <v>0.001369568682819718</v>
+        <v>0.0002447834666090372</v>
       </c>
       <c r="M35" s="3">
-        <v>0.001346952882563965</v>
+        <v>0.0002401368117972023</v>
       </c>
       <c r="N35" s="3">
-        <v>0.001322484406668366</v>
+        <v>0.0002353212284016688</v>
       </c>
       <c r="O35" s="3">
-        <v>0.001297618315766307</v>
+        <v>0.0002304214056858827</v>
       </c>
       <c r="P35" s="3">
-        <v>0.00127291961504111</v>
+        <v>0.0002258087102620249</v>
       </c>
       <c r="Q35" s="3">
-        <v>0.001248665584473509</v>
+        <v>0.0002214332426650852</v>
       </c>
       <c r="R35" s="3">
-        <v>0.001224089698116828</v>
+        <v>0.0002169689070602865</v>
       </c>
     </row>
     <row r="36" spans="1:18">
@@ -5779,7 +5771,7 @@
         <v>39</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C36" s="3" t="s">
         <v>44</v>
@@ -5788,46 +5780,46 @@
         <v>45</v>
       </c>
       <c r="E36" s="3">
-        <v>0.8997000000000001</v>
+        <v>0</v>
       </c>
       <c r="F36" s="3">
-        <v>0.95</v>
+        <v>0.001488258363077195</v>
       </c>
       <c r="G36" s="3">
-        <v>0.9448246413287567</v>
+        <v>0.001485758849681867</v>
       </c>
       <c r="H36" s="3">
-        <v>0.9399963657464822</v>
+        <v>0.001475691483837327</v>
       </c>
       <c r="I36" s="3">
-        <v>0.931889011718065</v>
+        <v>0.001461704234987219</v>
       </c>
       <c r="J36" s="3">
-        <v>0.9215473613256085</v>
+        <v>0.001444656999222126</v>
       </c>
       <c r="K36" s="3">
-        <v>0.9091771664417031</v>
+        <v>0.001424277548675483</v>
       </c>
       <c r="L36" s="3">
-        <v>0.8950638881772701</v>
+        <v>0.001401476504745729</v>
       </c>
       <c r="M36" s="3">
-        <v>0.8802999445329061</v>
+        <v>0.001378334016486979</v>
       </c>
       <c r="N36" s="3">
-        <v>0.8647727539234891</v>
+        <v>0.001353295598597051</v>
       </c>
       <c r="O36" s="3">
-        <v>0.848611529377848</v>
+        <v>0.001327850242528963</v>
       </c>
       <c r="P36" s="3">
-        <v>0.8324747634640352</v>
+        <v>0.001302576131107969</v>
       </c>
       <c r="Q36" s="3">
-        <v>0.816597050672448</v>
+        <v>0.001277757022319043</v>
       </c>
       <c r="R36" s="3">
-        <v>0.8007057086587224</v>
+        <v>0.001252608541872664</v>
       </c>
     </row>
     <row r="37" spans="1:18">
@@ -5835,7 +5827,7 @@
         <v>39</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C37" s="3" t="s">
         <v>44</v>
@@ -5844,46 +5836,46 @@
         <v>45</v>
       </c>
       <c r="E37" s="3">
-        <v>0</v>
+        <v>0.8997000000000001</v>
       </c>
       <c r="F37" s="3">
-        <v>0.001199472032299156</v>
+        <v>0.95</v>
       </c>
       <c r="G37" s="3">
-        <v>0.001192937613369395</v>
+        <v>0.9448246453840015</v>
       </c>
       <c r="H37" s="3">
-        <v>0.001186841422290268</v>
+        <v>0.93999677780447</v>
       </c>
       <c r="I37" s="3">
-        <v>0.001176605059750231</v>
+        <v>0.9318900035689611</v>
       </c>
       <c r="J37" s="3">
-        <v>0.001163547669841213</v>
+        <v>0.9215488192564274</v>
       </c>
       <c r="K37" s="3">
-        <v>0.001147929035317703</v>
+        <v>0.9091789513811799</v>
       </c>
       <c r="L37" s="3">
-        <v>0.001130109579989026</v>
+        <v>0.8950658819449289</v>
       </c>
       <c r="M37" s="3">
-        <v>0.001111468593159705</v>
+        <v>0.8803020571600484</v>
       </c>
       <c r="N37" s="3">
-        <v>0.001091863929079522</v>
+        <v>0.8647749195875583</v>
       </c>
       <c r="O37" s="3">
-        <v>0.001071458732395097</v>
+        <v>0.8486137035314995</v>
       </c>
       <c r="P37" s="3">
-        <v>0.001051084417231543</v>
+        <v>0.832476915522699</v>
       </c>
       <c r="Q37" s="3">
-        <v>0.001031037183094293</v>
+        <v>0.8165991608806186</v>
       </c>
       <c r="R37" s="3">
-        <v>0.001010972740672015</v>
+        <v>0.8007077644901518</v>
       </c>
     </row>
     <row r="38" spans="1:18">
@@ -5891,7 +5883,7 @@
         <v>39</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C38" s="3" t="s">
         <v>44</v>
@@ -5903,43 +5895,43 @@
         <v>0</v>
       </c>
       <c r="F38" s="3">
-        <v>0.01510034352922579</v>
+        <v>0.001227414202372625</v>
       </c>
       <c r="G38" s="3">
-        <v>0.01481940690542624</v>
+        <v>0.001220727566837898</v>
       </c>
       <c r="H38" s="3">
-        <v>0.01448260220303019</v>
+        <v>0.00121448988974917</v>
       </c>
       <c r="I38" s="3">
-        <v>0.01422398430654751</v>
+        <v>0.001204015816241705</v>
       </c>
       <c r="J38" s="3">
-        <v>0.01397444072222211</v>
+        <v>0.001190654851510592</v>
       </c>
       <c r="K38" s="3">
-        <v>0.0136745600200285</v>
+        <v>0.001174672797287906</v>
       </c>
       <c r="L38" s="3">
-        <v>0.01338727934733883</v>
+        <v>0.001156438500587774</v>
       </c>
       <c r="M38" s="3">
-        <v>0.01316600200275472</v>
+        <v>0.001137363418248508</v>
       </c>
       <c r="N38" s="3">
-        <v>0.01284746969623646</v>
+        <v>0.001117302124376225</v>
       </c>
       <c r="O38" s="3">
-        <v>0.01259356713306973</v>
+        <v>0.001096421591623784</v>
       </c>
       <c r="P38" s="3">
-        <v>0.01234950575452187</v>
+        <v>0.001075572620273597</v>
       </c>
       <c r="Q38" s="3">
-        <v>0.01211472427629902</v>
+        <v>0.001055058323905726</v>
       </c>
       <c r="R38" s="3">
-        <v>0.0118445073779429</v>
+        <v>0.001034526402194998</v>
       </c>
     </row>
     <row r="39" spans="1:18">
@@ -5947,7 +5939,7 @@
         <v>39</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C39" s="3" t="s">
         <v>44</v>
@@ -5959,43 +5951,43 @@
         <v>0</v>
       </c>
       <c r="F39" s="3">
-        <v>0</v>
+        <v>0.01545211193707492</v>
       </c>
       <c r="G39" s="3">
-        <v>0</v>
+        <v>0.01516463078475725</v>
       </c>
       <c r="H39" s="3">
-        <v>0</v>
+        <v>0.01481998008510367</v>
       </c>
       <c r="I39" s="3">
-        <v>0</v>
+        <v>0.01455533758358397</v>
       </c>
       <c r="J39" s="3">
-        <v>0</v>
+        <v>0.01429998078387197</v>
       </c>
       <c r="K39" s="3">
-        <v>0</v>
+        <v>0.01399311424344553</v>
       </c>
       <c r="L39" s="3">
-        <v>0</v>
+        <v>0.01369914125513785</v>
       </c>
       <c r="M39" s="3">
-        <v>0</v>
+        <v>0.01347270916827607</v>
       </c>
       <c r="N39" s="3">
-        <v>0</v>
+        <v>0.0131467565271081</v>
       </c>
       <c r="O39" s="3">
-        <v>0</v>
+        <v>0.01288693920443798</v>
       </c>
       <c r="P39" s="3">
-        <v>0</v>
+        <v>0.01263719232063104</v>
       </c>
       <c r="Q39" s="3">
-        <v>0</v>
+        <v>0.0123969415160563</v>
       </c>
       <c r="R39" s="3">
-        <v>0</v>
+        <v>0.01212042980937847</v>
       </c>
     </row>
     <row r="40" spans="1:18">
@@ -6003,7 +5995,7 @@
         <v>39</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C40" s="3" t="s">
         <v>44</v>
@@ -6059,7 +6051,7 @@
         <v>39</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C41" s="3" t="s">
         <v>44</v>
@@ -6115,10 +6107,10 @@
         <v>39</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>43</v>
+        <v>59</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>58</v>
+        <v>44</v>
       </c>
       <c r="D42" s="3" t="s">
         <v>45</v>
@@ -6127,43 +6119,43 @@
         <v>0</v>
       </c>
       <c r="F42" s="3">
-        <v>10564.23237621565</v>
+        <v>0</v>
       </c>
       <c r="G42" s="3">
-        <v>10564.23237621565</v>
+        <v>0</v>
       </c>
       <c r="H42" s="3">
-        <v>10564.23237621565</v>
+        <v>0</v>
       </c>
       <c r="I42" s="3">
-        <v>10564.23237621565</v>
+        <v>0</v>
       </c>
       <c r="J42" s="3">
-        <v>10564.23237621565</v>
+        <v>0</v>
       </c>
       <c r="K42" s="3">
-        <v>10564.23237621565</v>
+        <v>0</v>
       </c>
       <c r="L42" s="3">
-        <v>10564.23237621565</v>
+        <v>0</v>
       </c>
       <c r="M42" s="3">
-        <v>10564.23237621565</v>
+        <v>0</v>
       </c>
       <c r="N42" s="3">
-        <v>10564.23237621565</v>
+        <v>0</v>
       </c>
       <c r="O42" s="3">
-        <v>10564.23237621565</v>
+        <v>0</v>
       </c>
       <c r="P42" s="3">
-        <v>10564.23237621565</v>
+        <v>0</v>
       </c>
       <c r="Q42" s="3">
-        <v>10564.23237621565</v>
+        <v>0</v>
       </c>
       <c r="R42" s="3">
-        <v>10564.23237621565</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43" spans="1:18">
@@ -6171,7 +6163,7 @@
         <v>39</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C43" s="3" t="s">
         <v>58</v>
@@ -6183,43 +6175,43 @@
         <v>0</v>
       </c>
       <c r="F43" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="G43" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="H43" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="I43" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="J43" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="K43" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="L43" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="M43" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="N43" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="O43" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="P43" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="Q43" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="R43" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
     </row>
     <row r="44" spans="1:18">
@@ -6227,7 +6219,7 @@
         <v>39</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C44" s="3" t="s">
         <v>58</v>
@@ -6239,43 +6231,43 @@
         <v>0</v>
       </c>
       <c r="F44" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="G44" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="H44" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="I44" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="J44" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="K44" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="L44" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="M44" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="N44" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="O44" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="P44" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="Q44" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="R44" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
     </row>
     <row r="45" spans="1:18">
@@ -6283,7 +6275,7 @@
         <v>39</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C45" s="3" t="s">
         <v>58</v>
@@ -6295,43 +6287,43 @@
         <v>0</v>
       </c>
       <c r="F45" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="G45" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="H45" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="I45" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="J45" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="K45" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="L45" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="M45" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="N45" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="O45" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="P45" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="Q45" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="R45" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
     </row>
     <row r="46" spans="1:18">
@@ -6339,7 +6331,7 @@
         <v>39</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C46" s="3" t="s">
         <v>58</v>
@@ -6348,46 +6340,46 @@
         <v>45</v>
       </c>
       <c r="E46" s="3">
-        <v>3317810.965630114</v>
+        <v>0</v>
       </c>
       <c r="F46" s="3">
-        <v>7136539.752798174</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="G46" s="3">
-        <v>7136539.752798174</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="H46" s="3">
-        <v>7136539.752798174</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="I46" s="3">
-        <v>7136539.752798174</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="J46" s="3">
-        <v>7136539.752798174</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="K46" s="3">
-        <v>7136539.752798174</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="L46" s="3">
-        <v>7136539.752798174</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="M46" s="3">
-        <v>7136539.752798174</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="N46" s="3">
-        <v>7136539.752798174</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="O46" s="3">
-        <v>7136539.752798174</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="P46" s="3">
-        <v>7136539.752798174</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="Q46" s="3">
-        <v>7136539.752798174</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="R46" s="3">
-        <v>7136539.752798174</v>
+        <v>10810.33030080507</v>
       </c>
     </row>
     <row r="47" spans="1:18">
@@ -6395,7 +6387,7 @@
         <v>39</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C47" s="3" t="s">
         <v>58</v>
@@ -6404,46 +6396,46 @@
         <v>45</v>
       </c>
       <c r="E47" s="3">
-        <v>4095441.930000001</v>
+        <v>3317810.965630114</v>
       </c>
       <c r="F47" s="3">
-        <v>10564.23237621565</v>
+        <v>7134324.87147687</v>
       </c>
       <c r="G47" s="3">
-        <v>10564.23237621565</v>
+        <v>7134324.87147687</v>
       </c>
       <c r="H47" s="3">
-        <v>10564.23237621565</v>
+        <v>7134324.87147687</v>
       </c>
       <c r="I47" s="3">
-        <v>10564.23237621565</v>
+        <v>7134324.87147687</v>
       </c>
       <c r="J47" s="3">
-        <v>10564.23237621565</v>
+        <v>7134324.87147687</v>
       </c>
       <c r="K47" s="3">
-        <v>10564.23237621565</v>
+        <v>7134324.87147687</v>
       </c>
       <c r="L47" s="3">
-        <v>10564.23237621565</v>
+        <v>7134324.87147687</v>
       </c>
       <c r="M47" s="3">
-        <v>10564.23237621565</v>
+        <v>7134324.87147687</v>
       </c>
       <c r="N47" s="3">
-        <v>10564.23237621565</v>
+        <v>7134324.87147687</v>
       </c>
       <c r="O47" s="3">
-        <v>10564.23237621565</v>
+        <v>7134324.87147687</v>
       </c>
       <c r="P47" s="3">
-        <v>10564.23237621565</v>
+        <v>7134324.87147687</v>
       </c>
       <c r="Q47" s="3">
-        <v>10564.23237621565</v>
+        <v>7134324.87147687</v>
       </c>
       <c r="R47" s="3">
-        <v>10564.23237621565</v>
+        <v>7134324.87147687</v>
       </c>
     </row>
     <row r="48" spans="1:18">
@@ -6451,7 +6443,7 @@
         <v>39</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C48" s="3" t="s">
         <v>58</v>
@@ -6460,46 +6452,46 @@
         <v>45</v>
       </c>
       <c r="E48" s="3">
-        <v>0</v>
+        <v>4095441.930000001</v>
       </c>
       <c r="F48" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="G48" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="H48" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="I48" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="J48" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="K48" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="L48" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="M48" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="N48" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="O48" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="P48" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="Q48" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="R48" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
     </row>
     <row r="49" spans="1:18">
@@ -6507,7 +6499,7 @@
         <v>39</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C49" s="3" t="s">
         <v>58</v>
@@ -6519,43 +6511,43 @@
         <v>0</v>
       </c>
       <c r="F49" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="G49" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="H49" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="I49" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="J49" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="K49" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="L49" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="M49" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="N49" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="O49" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="P49" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="Q49" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="R49" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
     </row>
     <row r="50" spans="1:18">
@@ -6563,7 +6555,7 @@
         <v>39</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C50" s="3" t="s">
         <v>58</v>
@@ -6572,46 +6564,46 @@
         <v>45</v>
       </c>
       <c r="E50" s="3">
-        <v>3248848.027554</v>
+        <v>0</v>
       </c>
       <c r="F50" s="3">
-        <v>3430483.079</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="G50" s="3">
-        <v>3430483.079</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="H50" s="3">
-        <v>3430483.079</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="I50" s="3">
-        <v>3430483.079</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="J50" s="3">
-        <v>3430483.079</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="K50" s="3">
-        <v>3430483.079</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="L50" s="3">
-        <v>3430483.079</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="M50" s="3">
-        <v>3430483.079</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="N50" s="3">
-        <v>3430483.079</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="O50" s="3">
-        <v>3430483.079</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="P50" s="3">
-        <v>3430483.079</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="Q50" s="3">
-        <v>3430483.079</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="R50" s="3">
-        <v>3430483.079</v>
+        <v>10810.33030080507</v>
       </c>
     </row>
     <row r="51" spans="1:18">
@@ -6619,7 +6611,7 @@
         <v>39</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C51" s="3" t="s">
         <v>58</v>
@@ -6628,46 +6620,46 @@
         <v>45</v>
       </c>
       <c r="E51" s="3">
-        <v>0</v>
+        <v>3248848.027554</v>
       </c>
       <c r="F51" s="3">
-        <v>10564.23237621565</v>
+        <v>3430483.079</v>
       </c>
       <c r="G51" s="3">
-        <v>10564.23237621565</v>
+        <v>3430483.079</v>
       </c>
       <c r="H51" s="3">
-        <v>10564.23237621565</v>
+        <v>3430483.079</v>
       </c>
       <c r="I51" s="3">
-        <v>10564.23237621565</v>
+        <v>3430483.079</v>
       </c>
       <c r="J51" s="3">
-        <v>10564.23237621565</v>
+        <v>3430483.079</v>
       </c>
       <c r="K51" s="3">
-        <v>10564.23237621565</v>
+        <v>3430483.079</v>
       </c>
       <c r="L51" s="3">
-        <v>10564.23237621565</v>
+        <v>3430483.079</v>
       </c>
       <c r="M51" s="3">
-        <v>10564.23237621565</v>
+        <v>3430483.079</v>
       </c>
       <c r="N51" s="3">
-        <v>10564.23237621565</v>
+        <v>3430483.079</v>
       </c>
       <c r="O51" s="3">
-        <v>10564.23237621565</v>
+        <v>3430483.079</v>
       </c>
       <c r="P51" s="3">
-        <v>10564.23237621565</v>
+        <v>3430483.079</v>
       </c>
       <c r="Q51" s="3">
-        <v>10564.23237621565</v>
+        <v>3430483.079</v>
       </c>
       <c r="R51" s="3">
-        <v>10564.23237621565</v>
+        <v>3430483.079</v>
       </c>
     </row>
     <row r="52" spans="1:18">
@@ -6675,7 +6667,7 @@
         <v>39</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C52" s="3" t="s">
         <v>58</v>
@@ -6687,43 +6679,43 @@
         <v>0</v>
       </c>
       <c r="F52" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="G52" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="H52" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="I52" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="J52" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="K52" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="L52" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="M52" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="N52" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="O52" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="P52" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="Q52" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="R52" s="3">
-        <v>10564.23237621565</v>
+        <v>10810.33030080507</v>
       </c>
     </row>
     <row r="53" spans="1:18">
@@ -6731,7 +6723,7 @@
         <v>39</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C53" s="3" t="s">
         <v>58</v>
@@ -6743,43 +6735,43 @@
         <v>0</v>
       </c>
       <c r="F53" s="3">
-        <v>0</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="G53" s="3">
-        <v>0</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="H53" s="3">
-        <v>0</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="I53" s="3">
-        <v>0</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="J53" s="3">
-        <v>0</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="K53" s="3">
-        <v>0</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="L53" s="3">
-        <v>0</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="M53" s="3">
-        <v>0</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="N53" s="3">
-        <v>0</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="O53" s="3">
-        <v>0</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="P53" s="3">
-        <v>0</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="Q53" s="3">
-        <v>0</v>
+        <v>10810.33030080507</v>
       </c>
       <c r="R53" s="3">
-        <v>0</v>
+        <v>10810.33030080507</v>
       </c>
     </row>
     <row r="54" spans="1:18">
@@ -6787,7 +6779,7 @@
         <v>39</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C54" s="3" t="s">
         <v>58</v>
@@ -6843,7 +6835,7 @@
         <v>39</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C55" s="3" t="s">
         <v>58</v>
@@ -6893,6 +6885,78 @@
       <c r="R55" s="3">
         <v>0</v>
       </c>
+    </row>
+    <row r="56" spans="1:18">
+      <c r="A56" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B56" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C56" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="D56" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E56" s="3">
+        <v>0</v>
+      </c>
+      <c r="F56" s="3">
+        <v>0</v>
+      </c>
+      <c r="G56" s="3">
+        <v>0</v>
+      </c>
+      <c r="H56" s="3">
+        <v>0</v>
+      </c>
+      <c r="I56" s="3">
+        <v>0</v>
+      </c>
+      <c r="J56" s="3">
+        <v>0</v>
+      </c>
+      <c r="K56" s="3">
+        <v>0</v>
+      </c>
+      <c r="L56" s="3">
+        <v>0</v>
+      </c>
+      <c r="M56" s="3">
+        <v>0</v>
+      </c>
+      <c r="N56" s="3">
+        <v>0</v>
+      </c>
+      <c r="O56" s="3">
+        <v>0</v>
+      </c>
+      <c r="P56" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q56" s="3">
+        <v>0</v>
+      </c>
+      <c r="R56" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:18">
+      <c r="A57" s="2"/>
+      <c r="B57" s="3"/>
+      <c r="C57" s="3"/>
+      <c r="D57" s="3"/>
+      <c r="E57" s="3"/>
+      <c r="F57" s="3"/>
+      <c r="G57" s="3"/>
+      <c r="H57" s="3"/>
+      <c r="I57" s="3"/>
+      <c r="J57" s="3"/>
+      <c r="K57" s="3"/>
+      <c r="L57" s="3"/>
+      <c r="M57" s="3"/>
+      <c r="N57" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6901,7 +6965,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R19"/>
+  <dimension ref="A1:R21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
@@ -7465,60 +7529,20 @@
       </c>
     </row>
     <row r="11" spans="1:18">
-      <c r="A11" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="D11" s="3">
-        <v>0</v>
-      </c>
-      <c r="E11" s="3">
-        <v>85194803013.39064</v>
-      </c>
-      <c r="F11" s="3">
-        <v>84404890393.58084</v>
-      </c>
-      <c r="G11" s="3">
-        <v>84929115541.41525</v>
-      </c>
-      <c r="H11" s="3">
-        <v>85583117736.72563</v>
-      </c>
-      <c r="I11" s="3">
-        <v>86522529344.67421</v>
-      </c>
-      <c r="J11" s="3">
-        <v>87714644472.82254</v>
-      </c>
-      <c r="K11" s="3">
-        <v>89069505812.59819</v>
-      </c>
-      <c r="L11" s="3">
-        <v>90712749984.36397</v>
-      </c>
-      <c r="M11" s="3">
-        <v>92444828225.81683</v>
-      </c>
-      <c r="N11" s="3">
-        <v>94310890727.90857</v>
-      </c>
-      <c r="O11" s="3">
-        <v>96258719122.24478</v>
-      </c>
-      <c r="P11" s="3">
-        <v>98337635291.84836</v>
-      </c>
-      <c r="Q11" s="3">
-        <v>100422892085.2535</v>
-      </c>
-      <c r="R11" s="3">
-        <v>1175906321752.643</v>
-      </c>
+      <c r="A11" s="2"/>
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="3"/>
+      <c r="I11" s="3"/>
+      <c r="J11" s="3"/>
+      <c r="K11" s="3"/>
+      <c r="L11" s="3"/>
+      <c r="M11" s="3"/>
+      <c r="N11" s="3"/>
     </row>
     <row r="12" spans="1:18">
       <c r="A12" s="2" t="s">
@@ -7528,52 +7552,52 @@
         <v>9</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D12" s="3">
         <v>0</v>
       </c>
       <c r="E12" s="3">
-        <v>22719495997.45493</v>
+        <v>85194907200.1624</v>
       </c>
       <c r="F12" s="3">
-        <v>21589748846.89655</v>
+        <v>84405703445.01935</v>
       </c>
       <c r="G12" s="3">
-        <v>21951296446.34491</v>
+        <v>84930026932.77505</v>
       </c>
       <c r="H12" s="3">
-        <v>22348131950.14209</v>
+        <v>85584119654.26726</v>
       </c>
       <c r="I12" s="3">
-        <v>22807606219.78644</v>
+        <v>86523605501.65433</v>
       </c>
       <c r="J12" s="3">
-        <v>23299284255.63233</v>
+        <v>87715774446.02568</v>
       </c>
       <c r="K12" s="3">
-        <v>23763358443.0893</v>
+        <v>89070668636.80901</v>
       </c>
       <c r="L12" s="3">
-        <v>24335728575.61003</v>
+        <v>90713940702.26074</v>
       </c>
       <c r="M12" s="3">
-        <v>24877832515.91828</v>
+        <v>92446038492.73221</v>
       </c>
       <c r="N12" s="3">
-        <v>25439974138.43624</v>
+        <v>94312109892.65094</v>
       </c>
       <c r="O12" s="3">
-        <v>25994850413.06195</v>
+        <v>96259946005.18753</v>
       </c>
       <c r="P12" s="3">
-        <v>26610605289.7963</v>
+        <v>98338869784.3856</v>
       </c>
       <c r="Q12" s="3">
-        <v>27188818878.54765</v>
+        <v>100424129507.4878</v>
       </c>
       <c r="R12" s="3">
-        <v>312926731970.717</v>
+        <v>1175919840201.418</v>
       </c>
     </row>
     <row r="13" spans="1:18">
@@ -7584,52 +7608,52 @@
         <v>9</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D13" s="3">
         <v>0</v>
       </c>
       <c r="E13" s="3">
-        <v>2717746279.21142</v>
+        <v>22719502911.73457</v>
       </c>
       <c r="F13" s="3">
-        <v>2894317790.600573</v>
+        <v>21590480830.17635</v>
       </c>
       <c r="G13" s="3">
-        <v>2947735736.458499</v>
+        <v>21952026872.26524</v>
       </c>
       <c r="H13" s="3">
-        <v>2999228863.59578</v>
+        <v>22348857479.207</v>
       </c>
       <c r="I13" s="3">
-        <v>3064861924.15613</v>
+        <v>22808333227.51225</v>
       </c>
       <c r="J13" s="3">
-        <v>3131389146.821229</v>
+        <v>23300012920.92625</v>
       </c>
       <c r="K13" s="3">
-        <v>3183817120.098674</v>
+        <v>23764082830.96848</v>
       </c>
       <c r="L13" s="3">
-        <v>3261709964.96347</v>
+        <v>24336454003.6489</v>
       </c>
       <c r="M13" s="3">
-        <v>3329025840.756422</v>
+        <v>24878559924.9792</v>
       </c>
       <c r="N13" s="3">
-        <v>3393753743.501169</v>
+        <v>25440697249.9491</v>
       </c>
       <c r="O13" s="3">
-        <v>3459355425.14792</v>
+        <v>25995572400.97338</v>
       </c>
       <c r="P13" s="3">
-        <v>3538113632.307089</v>
+        <v>26611328655.05474</v>
       </c>
       <c r="Q13" s="3">
-        <v>3604485477.241018</v>
+        <v>27189541405.92036</v>
       </c>
       <c r="R13" s="3">
-        <v>41525540944.8594</v>
+        <v>312935450713.3158</v>
       </c>
     </row>
     <row r="14" spans="1:18">
@@ -7640,52 +7664,52 @@
         <v>9</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D14" s="3">
         <v>0</v>
       </c>
       <c r="E14" s="3">
-        <v>58905734197.09176</v>
+        <v>2717808297.706973</v>
       </c>
       <c r="F14" s="3">
-        <v>59056406256.72191</v>
+        <v>2894316473.285625</v>
       </c>
       <c r="G14" s="3">
-        <v>59147533631.09243</v>
+        <v>2947734132.85289</v>
       </c>
       <c r="H14" s="3">
-        <v>59336735606.577</v>
+        <v>2999227614.362074</v>
       </c>
       <c r="I14" s="3">
-        <v>59733848377.38585</v>
+        <v>3064860695.407766</v>
       </c>
       <c r="J14" s="3">
-        <v>60346106002.87461</v>
+        <v>3131387642.16954</v>
       </c>
       <c r="K14" s="3">
-        <v>61161592604.01636</v>
+        <v>3183815658.68891</v>
       </c>
       <c r="L14" s="3">
-        <v>62135251471.59244</v>
+        <v>3261708814.60484</v>
       </c>
       <c r="M14" s="3">
-        <v>63230910339.70621</v>
+        <v>3329024155.014235</v>
       </c>
       <c r="N14" s="3">
-        <v>64445881648.41473</v>
+        <v>3393752377.438707</v>
       </c>
       <c r="O14" s="3">
-        <v>65748804745.92617</v>
+        <v>3459354089.85299</v>
       </c>
       <c r="P14" s="3">
-        <v>67108842737.39155</v>
+        <v>3538112321.558228</v>
       </c>
       <c r="Q14" s="3">
-        <v>68521217410.90862</v>
+        <v>3604483944.081652</v>
       </c>
       <c r="R14" s="3">
-        <v>808878865029.6997</v>
+        <v>41525586217.02443</v>
       </c>
     </row>
     <row r="15" spans="1:18">
@@ -7696,52 +7720,52 @@
         <v>9</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D15" s="3">
         <v>0</v>
       </c>
       <c r="E15" s="3">
-        <v>568131735.502313</v>
+        <v>58905708062.92641</v>
       </c>
       <c r="F15" s="3">
-        <v>571238500.3556887</v>
+        <v>59056426705.28291</v>
       </c>
       <c r="G15" s="3">
-        <v>576808941.2864491</v>
+        <v>59147654888.58762</v>
       </c>
       <c r="H15" s="3">
-        <v>583844477.0589781</v>
+        <v>59336952276.16656</v>
       </c>
       <c r="I15" s="3">
-        <v>592351777.6998091</v>
+        <v>59734137822.82865</v>
       </c>
       <c r="J15" s="3">
-        <v>602186987.75893</v>
+        <v>60346448089.47074</v>
       </c>
       <c r="K15" s="3">
-        <v>612525816.6264801</v>
+        <v>61161972144.89671</v>
       </c>
       <c r="L15" s="3">
-        <v>623850089.6663957</v>
+        <v>62135657253.72447</v>
       </c>
       <c r="M15" s="3">
-        <v>635965134.8583637</v>
+        <v>63231334542.04784</v>
       </c>
       <c r="N15" s="3">
-        <v>648397591.4513019</v>
+        <v>64446318809.77946</v>
       </c>
       <c r="O15" s="3">
-        <v>661032895.3780229</v>
+        <v>65749250785.25061</v>
       </c>
       <c r="P15" s="3">
-        <v>674269156.7811122</v>
+        <v>67109294853.30429</v>
       </c>
       <c r="Q15" s="3">
-        <v>687759713.6863912</v>
+        <v>68521673766.12736</v>
       </c>
       <c r="R15" s="3">
-        <v>8038362818.110236</v>
+        <v>808882830000.3937</v>
       </c>
     </row>
     <row r="16" spans="1:18">
@@ -7752,52 +7776,52 @@
         <v>9</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D16" s="3">
         <v>0</v>
       </c>
       <c r="E16" s="3">
-        <v>385906549.1300633</v>
+        <v>568130693.6193159</v>
       </c>
       <c r="F16" s="3">
-        <v>394841285.339397</v>
+        <v>571237123.0121137</v>
       </c>
       <c r="G16" s="3">
-        <v>402178302.6803991</v>
+        <v>576807161.9389294</v>
       </c>
       <c r="H16" s="3">
-        <v>409300838.8005061</v>
+        <v>583842398.850714</v>
       </c>
       <c r="I16" s="3">
-        <v>418049158.487105</v>
+        <v>592349484.6981652</v>
       </c>
       <c r="J16" s="3">
-        <v>426958490.3009185</v>
+        <v>602184539.7651516</v>
       </c>
       <c r="K16" s="3">
-        <v>434239114.6789761</v>
+        <v>612523260.2295734</v>
       </c>
       <c r="L16" s="3">
-        <v>444606819.4734921</v>
+        <v>623847455.812422</v>
       </c>
       <c r="M16" s="3">
-        <v>453675678.9584904</v>
+        <v>635962444.2167403</v>
       </c>
       <c r="N16" s="3">
-        <v>462577564.6360836</v>
+        <v>648394862.3590575</v>
       </c>
       <c r="O16" s="3">
-        <v>471481797.9816924</v>
+        <v>661030140.507823</v>
       </c>
       <c r="P16" s="3">
-        <v>482009559.6614543</v>
+        <v>674266382.7712355</v>
       </c>
       <c r="Q16" s="3">
-        <v>491075211.3628312</v>
+        <v>687756926.2464501</v>
       </c>
       <c r="R16" s="3">
-        <v>5676900371.491409</v>
+        <v>8038332874.027692</v>
       </c>
     </row>
     <row r="17" spans="1:18">
@@ -7808,52 +7832,52 @@
         <v>9</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D17" s="3">
         <v>0</v>
       </c>
       <c r="E17" s="3">
-        <v>172991699.2167722</v>
+        <v>385908330.7421014</v>
       </c>
       <c r="F17" s="3">
-        <v>181254460.1370325</v>
+        <v>394842169.7920454</v>
       </c>
       <c r="G17" s="3">
-        <v>188458735.4417266</v>
+        <v>402179122.0942766</v>
       </c>
       <c r="H17" s="3">
-        <v>194861459.0214449</v>
+        <v>409301663.2532659</v>
       </c>
       <c r="I17" s="3">
-        <v>202137806.3348214</v>
+        <v>418049988.4018263</v>
       </c>
       <c r="J17" s="3">
-        <v>210169337.7256945</v>
+        <v>426959320.788592</v>
       </c>
       <c r="K17" s="3">
-        <v>217289197.7445626</v>
+        <v>434239943.9731245</v>
       </c>
       <c r="L17" s="3">
-        <v>225498446.4254824</v>
+        <v>444607656.102468</v>
       </c>
       <c r="M17" s="3">
-        <v>234218341.9755156</v>
+        <v>453676511.1954297</v>
       </c>
       <c r="N17" s="3">
-        <v>242214607.3852603</v>
+        <v>462578399.4663827</v>
       </c>
       <c r="O17" s="3">
-        <v>250216046.1426421</v>
+        <v>471482632.8493508</v>
       </c>
       <c r="P17" s="3">
-        <v>259177474.5817247</v>
+        <v>482010397.3587667</v>
       </c>
       <c r="Q17" s="3">
-        <v>267815794.8797937</v>
+        <v>491076046.1881998</v>
       </c>
       <c r="R17" s="3">
-        <v>2846303407.012473</v>
+        <v>5676912182.20583</v>
       </c>
     </row>
     <row r="18" spans="1:18">
@@ -7864,52 +7888,52 @@
         <v>9</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D18" s="3">
         <v>0</v>
       </c>
       <c r="E18" s="3">
-        <v>496545126.0286096</v>
+        <v>173043771.6819614</v>
       </c>
       <c r="F18" s="3">
-        <v>506699065.0663942</v>
+        <v>181306519.6038624</v>
       </c>
       <c r="G18" s="3">
-        <v>519391488.8636248</v>
+        <v>188510506.5703169</v>
       </c>
       <c r="H18" s="3">
-        <v>529545427.9014096</v>
+        <v>194913190.6244135</v>
       </c>
       <c r="I18" s="3">
-        <v>539699366.9391943</v>
+        <v>202189722.5845824</v>
       </c>
       <c r="J18" s="3">
-        <v>552391790.736425</v>
+        <v>210221202.9508957</v>
       </c>
       <c r="K18" s="3">
-        <v>565084214.533656</v>
+        <v>217340801.1300305</v>
       </c>
       <c r="L18" s="3">
-        <v>575238153.5714406</v>
+        <v>225550435.7329436</v>
       </c>
       <c r="M18" s="3">
-        <v>590469062.1281174</v>
+        <v>234270066.9032318</v>
       </c>
       <c r="N18" s="3">
-        <v>603161485.9253483</v>
+        <v>242266290.0338671</v>
       </c>
       <c r="O18" s="3">
-        <v>615853909.7225791</v>
+        <v>250267687.6856053</v>
       </c>
       <c r="P18" s="3">
-        <v>628546333.51981</v>
+        <v>259229269.166969</v>
       </c>
       <c r="Q18" s="3">
-        <v>643777242.0764873</v>
+        <v>267867350.7598268</v>
       </c>
       <c r="R18" s="3">
-        <v>7366402667.013096</v>
+        <v>2846976815.428506</v>
       </c>
     </row>
     <row r="19" spans="1:18">
@@ -7920,53 +7944,125 @@
         <v>9</v>
       </c>
       <c r="C19" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="D19" s="3">
+        <v>0</v>
+      </c>
+      <c r="E19" s="3">
+        <v>496557253.3117262</v>
+      </c>
+      <c r="F19" s="3">
+        <v>506711192.349511</v>
+      </c>
+      <c r="G19" s="3">
+        <v>519403616.1467419</v>
+      </c>
+      <c r="H19" s="3">
+        <v>529557555.1845265</v>
+      </c>
+      <c r="I19" s="3">
+        <v>539711494.222311</v>
+      </c>
+      <c r="J19" s="3">
+        <v>552403918.0195417</v>
+      </c>
+      <c r="K19" s="3">
+        <v>565096341.8167726</v>
+      </c>
+      <c r="L19" s="3">
+        <v>575250280.8545572</v>
+      </c>
+      <c r="M19" s="3">
+        <v>590481189.4112341</v>
+      </c>
+      <c r="N19" s="3">
+        <v>603173613.208465</v>
+      </c>
+      <c r="O19" s="3">
+        <v>615866037.0056958</v>
+      </c>
+      <c r="P19" s="3">
+        <v>628558460.8029268</v>
+      </c>
+      <c r="Q19" s="3">
+        <v>643789369.3596038</v>
+      </c>
+      <c r="R19" s="3">
+        <v>7366560321.693613</v>
+      </c>
+    </row>
+    <row r="20" spans="1:18">
+      <c r="A20" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C20" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="D19" s="3">
-        <v>0</v>
-      </c>
-      <c r="E19" s="3">
-        <v>64528.01488962576</v>
-      </c>
-      <c r="F19" s="3">
-        <v>66759.14210145974</v>
-      </c>
-      <c r="G19" s="3">
-        <v>68864.60800164791</v>
-      </c>
-      <c r="H19" s="3">
-        <v>70791.22944198454</v>
-      </c>
-      <c r="I19" s="3">
-        <v>73030.85905438749</v>
-      </c>
-      <c r="J19" s="3">
-        <v>75441.57424663815</v>
-      </c>
-      <c r="K19" s="3">
-        <v>77531.16812264835</v>
-      </c>
-      <c r="L19" s="3">
-        <v>80102.00821263029</v>
-      </c>
-      <c r="M19" s="3">
-        <v>82669.43243499412</v>
-      </c>
-      <c r="N19" s="3">
-        <v>85077.43058664071</v>
-      </c>
-      <c r="O19" s="3">
-        <v>87484.8471815134</v>
-      </c>
-      <c r="P19" s="3">
-        <v>90227.13223671311</v>
-      </c>
-      <c r="Q19" s="3">
-        <v>92779.27641959638</v>
-      </c>
-      <c r="R19" s="3">
-        <v>1015286.72293048</v>
-      </c>
+      <c r="D20" s="3">
+        <v>0</v>
+      </c>
+      <c r="E20" s="3">
+        <v>64539.92354682603</v>
+      </c>
+      <c r="F20" s="3">
+        <v>66771.10099528854</v>
+      </c>
+      <c r="G20" s="3">
+        <v>68876.50759517669</v>
+      </c>
+      <c r="H20" s="3">
+        <v>70803.12524100012</v>
+      </c>
+      <c r="I20" s="3">
+        <v>73042.80245124461</v>
+      </c>
+      <c r="J20" s="3">
+        <v>75453.51214357962</v>
+      </c>
+      <c r="K20" s="3">
+        <v>77543.05164529754</v>
+      </c>
+      <c r="L20" s="3">
+        <v>80113.98507624693</v>
+      </c>
+      <c r="M20" s="3">
+        <v>82681.35516281333</v>
+      </c>
+      <c r="N20" s="3">
+        <v>85089.34865779919</v>
+      </c>
+      <c r="O20" s="3">
+        <v>87496.76077650186</v>
+      </c>
+      <c r="P20" s="3">
+        <v>90239.08596337376</v>
+      </c>
+      <c r="Q20" s="3">
+        <v>92791.18075274017</v>
+      </c>
+      <c r="R20" s="3">
+        <v>1015441.740007888</v>
+      </c>
+    </row>
+    <row r="21" spans="1:18">
+      <c r="A21" s="2"/>
+      <c r="B21" s="3"/>
+      <c r="C21" s="3"/>
+      <c r="D21" s="3"/>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="3"/>
+      <c r="I21" s="3"/>
+      <c r="J21" s="3"/>
+      <c r="K21" s="3"/>
+      <c r="L21" s="3"/>
+      <c r="M21" s="3"/>
+      <c r="N21" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>